<commit_message>
07.01.01: Excel del CEO actualizado, olvidado en a16f4ef
El commit a16f4ef dio una lista de ficheros y omitio el Excel de
05-vista-ceo/. La version que quedo en git enseñaba las 29 reglas
derogadas por D-16; esta es la regenerada tras la revision transversal
02.03.01 y la correccion 03.01.13. verificar_excel.py: sin fallos, 1
aviso conocido (07.01.01, 4 marcas en negrita), censo 54 tareas / 13
hechas.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/05-vista-ceo/WBS_Bot_Trading_v0.9.xlsx
+++ b/05-vista-ceo/WBS_Bot_Trading_v0.9.xlsx
@@ -674,7 +674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -1078,12 +1078,12 @@
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
         <is>
-          <t>02.03.01</t>
+          <t>03.01.08</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Revisión independiente de método, fuentes y números</t>
+          <t>Prueba de fuego de las barreras (regla 25 de CLAUDE.md): inyectar cada caso prohibido —leer el cajón reservado, escribir fuera del proyecto, borrar datos, gastar dinero— y comprobar que se bloquea de verdad. Lo que no se bloquee se marca "no verificada"</t>
         </is>
       </c>
       <c r="C18" s="4" t="n"/>
@@ -1099,12 +1099,12 @@
     <row r="19">
       <c r="A19" s="13" t="inlineStr">
         <is>
-          <t>03.01.08</t>
+          <t>03.01.11</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Prueba de fuego de las barreras (regla 25 de CLAUDE.md): inyectar cada caso prohibido —leer el cajón reservado, escribir fuera del proyecto, borrar datos, gastar dinero— y comprobar que se bloquea de verdad. Lo que no se bloquee se marca "no verificada"</t>
+          <t>NUEVA 31/07 (D-10): guardia del cajon reservado por cifrado. Script cajon_reservado.py: la contraseña solo la tiene el CEO, no se guarda, se pide en cada operacion y nada se descifra a disco</t>
         </is>
       </c>
       <c r="C19" s="4" t="n"/>
@@ -1117,109 +1117,87 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="13" t="inlineStr">
-        <is>
-          <t>03.01.11</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>NUEVA 31/07 (D-10): guardia del cajon reservado por cifrado. Script cajon_reservado.py: la contraseña solo la tiene el CEO, no se guarda, se pide en cada operacion y nada se descifra a disco</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="n"/>
-      <c r="D20" s="4" t="n"/>
-      <c r="E20" s="4" t="n"/>
-      <c r="F20" s="4" t="n"/>
-      <c r="G20" s="14" t="inlineStr">
-        <is>
-          <t>En curso</t>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>PROXIMA PUERTA</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>G1 — elegir mercado y tamaño de vela (criterios en la hoja PUERTAS)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>PROXIMA PUERTA</t>
+          <t>OBJETIVO DEL MES</t>
         </is>
       </c>
       <c r="B22" s="16" t="inlineStr">
         <is>
-          <t>G1 — elegir mercado y tamaño de vela (criterios en la hoja PUERTAS)</t>
+          <t>Llegar al 1 de septiembre con respuesta a: ¿existe alguna estrategia que merezca pasar a demo?</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>OBJETIVO DEL MES</t>
+          <t>FUENTE DE VERDAD</t>
         </is>
       </c>
       <c r="B23" s="16" t="inlineStr">
         <is>
-          <t>Llegar al 1 de septiembre con respuesta a: ¿existe alguna estrategia que merezca pasar a demo?</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="15" t="inlineStr">
-        <is>
-          <t>FUENTE DE VERDAD</t>
-        </is>
-      </c>
-      <c r="B24" s="16" t="inlineStr">
-        <is>
           <t>00-direccion/WBS.md — este Excel se genera de ahi. Si discrepan, manda el texto.</t>
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="15" t="inlineStr">
+        <is>
+          <t>LEYENDA</t>
+        </is>
+      </c>
+    </row>
     <row r="28">
-      <c r="A28" s="15" t="inlineStr">
-        <is>
-          <t>LEYENDA</t>
+      <c r="A28" s="17" t="inlineStr">
+        <is>
+          <t>Hecha</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="17" t="inlineStr">
-        <is>
-          <t>Hecha</t>
+      <c r="A29" s="18" t="inlineStr">
+        <is>
+          <t>En curso</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="18" t="inlineStr">
-        <is>
-          <t>En curso</t>
+      <c r="A30" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="20" t="inlineStr">
+      <c r="A31" s="20" t="inlineStr">
         <is>
           <t>Bloqueada</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="B24:G24"/>
+  <mergeCells count="10">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="B22:G22"/>
     <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B22:G22"/>
     <mergeCell ref="B23:G23"/>
     <mergeCell ref="B19:F19"/>
     <mergeCell ref="B14:F14"/>
+    <mergeCell ref="B21:G21"/>
     <mergeCell ref="B17:F17"/>
     <mergeCell ref="B18:F18"/>
   </mergeCells>
@@ -1776,7 +1754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I54"/>
+  <dimension ref="A1:I53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1829,7 +1807,7 @@
       <c r="B4" s="24" t="n"/>
       <c r="C4" s="25" t="inlineStr">
         <is>
-          <t>02.03.01 — Revisión independiente de método, fuentes y números</t>
+          <t>01.02.03 — Auditar el catálogo awesome-claude-code y, por ampliación del CEO (01/08), las fuentes oficiales de Anthropic y los mecanismos nativos de Claude Code; proponer máximo 4 piezas concretas para el motor, con motivo y coste de integración. Carril de motor: cuenta contra el 20% y se limita a 1 tirada</t>
         </is>
       </c>
       <c r="D4" s="24" t="n"/>
@@ -1839,7 +1817,7 @@
       <c r="H4" s="24" t="n"/>
       <c r="I4" s="25" t="inlineStr">
         <is>
-          <t>Orquestador</t>
+          <t>Investigador</t>
         </is>
       </c>
     </row>
@@ -1875,7 +1853,7 @@
       <c r="B6" s="30" t="n"/>
       <c r="C6" s="31" t="inlineStr">
         <is>
-          <t>02.03.01 — Revisión independiente de método, fuentes y números. Detras de ella esperan 18 de las 42 tareas vivas.</t>
+          <t>02.03.02 — Informe de decisión: 3-5 mercados poco correlacionados + 1-2 velas. Detras de ella esperan 17 de las 41 tareas vivas.</t>
         </is>
       </c>
       <c r="D6" s="30" t="n"/>
@@ -1994,22 +1972,22 @@
       </c>
       <c r="B11" s="33" t="inlineStr">
         <is>
-          <t>02.03.01</t>
+          <t>01.02.03</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Revisión independiente de método, fuentes y números</t>
+          <t>Auditar el catálogo awesome-claude-code y, por ampliación del CEO (01/08), las fuentes oficiales de Anthropic y los mecanismos nativos de Claude Code; proponer máximo 4 piezas concretas para el motor, con motivo y coste de integración. Carril de motor: cuenta contra el 20% y se limita a 1 tirada</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Orquestador</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>PRODUCTO</t>
+          <t>Investigador</t>
+        </is>
+      </c>
+      <c r="E11" s="34" t="inlineStr">
+        <is>
+          <t>MOTOR</t>
         </is>
       </c>
       <c r="F11" s="14" t="inlineStr">
@@ -2017,12 +1995,8 @@
           <t>En curso</t>
         </is>
       </c>
-      <c r="G11" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H11" s="5" t="n">
-        <v>18</v>
-      </c>
+      <c r="G11" s="5" t="inlineStr"/>
+      <c r="H11" s="5" t="inlineStr"/>
       <c r="I11" s="4" t="inlineStr">
         <is>
           <t>nada: se puede empezar ya</t>
@@ -2035,12 +2009,12 @@
       </c>
       <c r="B12" s="33" t="inlineStr">
         <is>
-          <t>01.02.03</t>
+          <t>01.02.04</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Auditar el catálogo awesome-claude-code y, por ampliación del CEO (01/08), las fuentes oficiales de Anthropic y los mecanismos nativos de Claude Code; proponer máximo 4 piezas concretas para el motor, con motivo y coste de integración. Carril de motor: cuenta contra el 20% y se limita a 1 tirada</t>
+          <t>NUEVA 01/08 (petición del CEO): evaluar si merece la pena añadir servidores MCP al proyecto, con veredicto por servidor y regla de admisión escrita para el futuro. Carril de motor: cuenta contra el 20% y se limita a 1 tirada</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -2072,27 +2046,27 @@
       </c>
       <c r="B13" s="33" t="inlineStr">
         <is>
-          <t>01.02.04</t>
+          <t>01.02.02</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>NUEVA 01/08 (petición del CEO): evaluar si merece la pena añadir servidores MCP al proyecto, con veredicto por servidor y regla de admisión escrita para el futuro. Carril de motor: cuenta contra el 20% y se limita a 1 tirada</t>
+          <t>Trasplante pieza a pieza desde gb2 (D6=B). Una tarea por pieza, cada una con su criterio de aceptación (ver sección Trasplante). Ninguna entra sin pasar su prueba ejecutada</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Investigador</t>
-        </is>
-      </c>
-      <c r="E13" s="34" t="inlineStr">
-        <is>
-          <t>MOTOR</t>
-        </is>
-      </c>
-      <c r="F13" s="14" t="inlineStr">
-        <is>
-          <t>En curso</t>
+          <t>Crítico + Constructores</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>PRODUCTO</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr"/>
@@ -2109,17 +2083,17 @@
       </c>
       <c r="B14" s="33" t="inlineStr">
         <is>
-          <t>01.02.02</t>
+          <t>02.01.01</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Trasplante pieza a pieza desde gb2 (D6=B). Una tarea por pieza, cada una con su criterio de aceptación (ver sección Trasplante). Ninguna entra sin pasar su prueba ejecutada</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>Crítico + Constructores</t>
+          <t>Confirmar 8 candidatos: EURUSD, GBPUSD, USDJPY, AUDUSD, USDCHF, XAUUSD, BTC, ETH</t>
+        </is>
+      </c>
+      <c r="D14" s="28" t="inlineStr">
+        <is>
+          <t>CEO + Orquestador</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -2146,17 +2120,17 @@
       </c>
       <c r="B15" s="33" t="inlineStr">
         <is>
-          <t>02.01.01</t>
+          <t>02.03.02</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Confirmar 8 candidatos: EURUSD, GBPUSD, USDJPY, AUDUSD, USDCHF, XAUUSD, BTC, ETH</t>
-        </is>
-      </c>
-      <c r="D15" s="28" t="inlineStr">
-        <is>
-          <t>CEO + Orquestador</t>
+          <t>Informe de decisión: 3-5 mercados poco correlacionados + 1-2 velas</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Orquestador</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -2169,8 +2143,12 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr"/>
-      <c r="H15" s="5" t="inlineStr"/>
+      <c r="G15" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>17</v>
+      </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
           <t>nada: se puede empezar ya</t>
@@ -2603,7 +2581,7 @@
     <row r="27">
       <c r="A27" s="32" t="inlineStr">
         <is>
-          <t>ESPERANDO A OTRA TAREA — 25 tareas, en orden de codigo WBS</t>
+          <t>ESPERANDO A OTRA TAREA — 24 tareas, en orden de codigo WBS</t>
         </is>
       </c>
       <c r="B27" s="32" t="n"/>
@@ -2623,17 +2601,17 @@
       </c>
       <c r="B28" s="33" t="inlineStr">
         <is>
-          <t>02.03.02</t>
+          <t>02.03.03</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Informe de decisión: 3-5 mercados poco correlacionados + 1-2 velas</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>Orquestador</t>
+          <t>PUERTA G1: el CEO elige</t>
+        </is>
+      </c>
+      <c r="D28" s="28" t="inlineStr">
+        <is>
+          <t>CEO</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -2650,11 +2628,11 @@
         <v>1</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>02.03.01 (en curso, Orquestador)</t>
+          <t>02.03.02 (pendiente, Orquestador)</t>
         </is>
       </c>
     </row>
@@ -2666,22 +2644,22 @@
       </c>
       <c r="B29" s="33" t="inlineStr">
         <is>
-          <t>02.03.03</t>
+          <t>03.01.05</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>PUERTA G1: el CEO elige</t>
-        </is>
-      </c>
-      <c r="D29" s="28" t="inlineStr">
-        <is>
-          <t>CEO</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>PRODUCTO</t>
+          <t>PRUEBA REAL DEL MOTOR: un día entero de trabajo desatendido de verdad antes de dar la fase por buena</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Orquestador</t>
+        </is>
+      </c>
+      <c r="E29" s="34" t="inlineStr">
+        <is>
+          <t>MOTOR</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
@@ -2689,15 +2667,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="G29" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H29" s="5" t="n">
-        <v>16</v>
-      </c>
+      <c r="G29" s="5" t="inlineStr"/>
+      <c r="H29" s="5" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>02.03.02 (pendiente, Orquestador)</t>
+          <t>03.01.03 (pendiente, Constructores), 03.01.04 (pendiente, Constructores)</t>
         </is>
       </c>
     </row>
@@ -2709,17 +2683,17 @@
       </c>
       <c r="B30" s="33" t="inlineStr">
         <is>
-          <t>03.01.05</t>
+          <t>03.01.07</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>PRUEBA REAL DEL MOTOR: un día entero de trabajo desatendido de verdad antes de dar la fase por buena</t>
+          <t>Cola de aprobación del CEO: tabla con desplegable Aprobado / Saltar / Corregir y columna de corrección. Lo aprobado se ejecuta solo; lo corregido se rehace Y la corrección se guarda en LECCIONES.md</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Orquestador</t>
+          <t>Secretario</t>
         </is>
       </c>
       <c r="E30" s="34" t="inlineStr">
@@ -2736,7 +2710,7 @@
       <c r="H30" s="5" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>03.01.03 (pendiente, Constructores), 03.01.04 (pendiente, Constructores)</t>
+          <t>03.01.06 (pendiente, Secretario)</t>
         </is>
       </c>
     </row>
@@ -2748,17 +2722,17 @@
       </c>
       <c r="B31" s="33" t="inlineStr">
         <is>
-          <t>03.01.07</t>
+          <t>03.01.08</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Cola de aprobación del CEO: tabla con desplegable Aprobado / Saltar / Corregir y columna de corrección. Lo aprobado se ejecuta solo; lo corregido se rehace Y la corrección se guarda en LECCIONES.md</t>
+          <t>Prueba de fuego de las barreras (regla 25 de CLAUDE.md): inyectar cada caso prohibido —leer el cajón reservado, escribir fuera del proyecto, borrar datos, gastar dinero— y comprobar que se bloquea de verdad. Lo que no se bloquee se marca "no verificada"</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Secretario</t>
+          <t>Crítico</t>
         </is>
       </c>
       <c r="E31" s="34" t="inlineStr">
@@ -2766,16 +2740,20 @@
           <t>MOTOR</t>
         </is>
       </c>
-      <c r="F31" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G31" s="5" t="inlineStr"/>
-      <c r="H31" s="5" t="inlineStr"/>
+      <c r="F31" s="14" t="inlineStr">
+        <is>
+          <t>En curso</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H31" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>03.01.06 (pendiente, Secretario)</t>
+          <t>03.01.03 (pendiente, Constructores)</t>
         </is>
       </c>
     </row>
@@ -2787,17 +2765,17 @@
       </c>
       <c r="B32" s="33" t="inlineStr">
         <is>
-          <t>03.01.08</t>
+          <t>03.01.11</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Prueba de fuego de las barreras (regla 25 de CLAUDE.md): inyectar cada caso prohibido —leer el cajón reservado, escribir fuera del proyecto, borrar datos, gastar dinero— y comprobar que se bloquea de verdad. Lo que no se bloquee se marca "no verificada"</t>
+          <t>NUEVA 31/07 (D-10): guardia del cajon reservado por cifrado. Script cajon_reservado.py: la contraseña solo la tiene el CEO, no se guarda, se pide en cada operacion y nada se descifra a disco</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Crítico</t>
+          <t>Constructores</t>
         </is>
       </c>
       <c r="E32" s="34" t="inlineStr">
@@ -2810,15 +2788,11 @@
           <t>En curso</t>
         </is>
       </c>
-      <c r="G32" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H32" s="5" t="n">
-        <v>1</v>
-      </c>
+      <c r="G32" s="5" t="inlineStr"/>
+      <c r="H32" s="5" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>03.01.03 (pendiente, Constructores)</t>
+          <t>03.01.08 (en curso, Crítico)</t>
         </is>
       </c>
     </row>
@@ -2830,34 +2804,38 @@
       </c>
       <c r="B33" s="33" t="inlineStr">
         <is>
-          <t>03.01.11</t>
+          <t>04.01.01</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>NUEVA 31/07 (D-10): guardia del cajon reservado por cifrado. Script cajon_reservado.py: la contraseña solo la tiene el CEO, no se guarda, se pide en cada operacion y nada se descifra a disco</t>
-        </is>
-      </c>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>Constructores</t>
-        </is>
-      </c>
-      <c r="E33" s="34" t="inlineStr">
-        <is>
-          <t>MOTOR</t>
-        </is>
-      </c>
-      <c r="F33" s="14" t="inlineStr">
-        <is>
-          <t>En curso</t>
-        </is>
-      </c>
-      <c r="G33" s="5" t="inlineStr"/>
-      <c r="H33" s="5" t="inlineStr"/>
+          <t>Comparar 3-4 brokers del mercado elegido; elegir uno y abrir demo (CEO firma)</t>
+        </is>
+      </c>
+      <c r="D33" s="28" t="inlineStr">
+        <is>
+          <t>CEO + Orquestador</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>PRODUCTO</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H33" s="5" t="n">
+        <v>15</v>
+      </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>03.01.08 (en curso, Crítico)</t>
+          <t>02.03.03 (pendiente, CEO)</t>
         </is>
       </c>
     </row>
@@ -2869,17 +2847,17 @@
       </c>
       <c r="B34" s="33" t="inlineStr">
         <is>
-          <t>04.01.01</t>
+          <t>04.01.02</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Comparar 3-4 brokers del mercado elegido; elegir uno y abrir demo (CEO firma)</t>
-        </is>
-      </c>
-      <c r="D34" s="28" t="inlineStr">
-        <is>
-          <t>CEO + Orquestador</t>
+          <t>Recalcular costes con precios reales del broker (sustituye 02.01.02)</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>Constructor datos</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -2892,15 +2870,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="G34" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="H34" s="5" t="n">
-        <v>15</v>
-      </c>
+      <c r="G34" s="5" t="inlineStr"/>
+      <c r="H34" s="5" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>02.03.03 (pendiente, CEO)</t>
+          <t>04.01.01 (pendiente, CEO + Orquestador)</t>
         </is>
       </c>
     </row>
@@ -2912,12 +2886,12 @@
       </c>
       <c r="B35" s="33" t="inlineStr">
         <is>
-          <t>04.01.02</t>
+          <t>04.01.03</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Recalcular costes con precios reales del broker (sustituye 02.01.02)</t>
+          <t>Histórico limpio partido en 3 cajones: construir (train), ajustar (validación) y RESERVADO bajo llave (OOS, se abre una sola vez por variante). Ningún agente toca el reservado</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -2935,8 +2909,12 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="G35" s="5" t="inlineStr"/>
-      <c r="H35" s="5" t="inlineStr"/>
+      <c r="G35" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H35" s="5" t="n">
+        <v>13</v>
+      </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
           <t>04.01.01 (pendiente, CEO + Orquestador)</t>
@@ -2951,17 +2929,17 @@
       </c>
       <c r="B36" s="33" t="inlineStr">
         <is>
-          <t>04.01.03</t>
+          <t>04.02.02</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Histórico limpio partido en 3 cajones: construir (train), ajustar (validación) y RESERVADO bajo llave (OOS, se abre una sola vez por variante). Ningún agente toca el reservado</t>
+          <t>Ficha por hipótesis: por qué existiría la ventaja, reglas de entrada/salida, mercado y vela. Sin lógica de por qué gana, no entra (nada de probar por probar)</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Constructor datos</t>
+          <t>Investigador</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -2978,11 +2956,11 @@
         <v>1</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>04.01.01 (pendiente, CEO + Orquestador)</t>
+          <t>04.02.01 (pendiente, Investigador)</t>
         </is>
       </c>
     </row>
@@ -2994,17 +2972,17 @@
       </c>
       <c r="B37" s="33" t="inlineStr">
         <is>
-          <t>04.02.02</t>
+          <t>04.02.03</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Ficha por hipótesis: por qué existiría la ventaja, reglas de entrada/salida, mercado y vela. Sin lógica de por qué gana, no entra (nada de probar por probar)</t>
+          <t>Filtro de sentido: el Validador puntúa y se eligen las 3-5 mejores</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Investigador</t>
+          <t>Validador</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -3021,11 +2999,11 @@
         <v>1</v>
       </c>
       <c r="H37" s="5" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>04.02.01 (pendiente, Investigador)</t>
+          <t>04.02.02 (pendiente, Investigador)</t>
         </is>
       </c>
     </row>
@@ -3037,12 +3015,12 @@
       </c>
       <c r="B38" s="33" t="inlineStr">
         <is>
-          <t>04.02.03</t>
+          <t>04.02.04</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Filtro de sentido: el Validador puntúa y se eligen las 3-5 mejores</t>
+          <t>Pre-registro de variantes: cada hipótesis deja escritas sus variantes ANTES de probar (máx. 5-7 por hipótesis). Lo no registrado no se prueba</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
@@ -3064,11 +3042,11 @@
         <v>1</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>04.02.02 (pendiente, Investigador)</t>
+          <t>04.02.03 (pendiente, Validador)</t>
         </is>
       </c>
     </row>
@@ -3080,17 +3058,17 @@
       </c>
       <c r="B39" s="33" t="inlineStr">
         <is>
-          <t>04.02.04</t>
+          <t>04.03.01</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Pre-registro de variantes: cada hipótesis deja escritas sus variantes ANTES de probar (máx. 5-7 por hipótesis). Lo no registrado no se prueba</t>
+          <t>Backtest con costes reales sobre el cajón de construir</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Validador</t>
+          <t>Constructores</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -3107,11 +3085,11 @@
         <v>1</v>
       </c>
       <c r="H39" s="5" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>04.02.03 (pendiente, Validador)</t>
+          <t>04.01.03 (pendiente, Constructor datos), 04.02.04 (pendiente, Validador)</t>
         </is>
       </c>
     </row>
@@ -3123,12 +3101,12 @@
       </c>
       <c r="B40" s="33" t="inlineStr">
         <is>
-          <t>04.03.01</t>
+          <t>04.03.02</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Backtest con costes reales sobre el cajón de construir</t>
+          <t>Ajuste SOLO con el cajón de validación; lo que no aguanta, muere aquí</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -3150,11 +3128,11 @@
         <v>1</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>04.01.03 (pendiente, Constructor datos), 04.02.04 (pendiente, Validador)</t>
+          <t>04.03.01 (pendiente, Constructores)</t>
         </is>
       </c>
     </row>
@@ -3166,17 +3144,17 @@
       </c>
       <c r="B41" s="33" t="inlineStr">
         <is>
-          <t>04.03.02</t>
+          <t>04.03.03</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Ajuste SOLO con el cajón de validación; lo que no aguanta, muere aquí</t>
+          <t>Prueba de fuego: UNA sola pasada por variante sobre el cajón reservado (OOS). Repetir sería hacerse trampa</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Constructores</t>
+          <t>Validador</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -3193,11 +3171,11 @@
         <v>1</v>
       </c>
       <c r="H41" s="5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>04.03.01 (pendiente, Constructores)</t>
+          <t>04.03.02 (pendiente, Constructores)</t>
         </is>
       </c>
     </row>
@@ -3209,12 +3187,12 @@
       </c>
       <c r="B42" s="33" t="inlineStr">
         <is>
-          <t>04.03.03</t>
+          <t>04.03.04</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Prueba de fuego: UNA sola pasada por variante sobre el cajón reservado (OOS). Repetir sería hacerse trampa</t>
+          <t>Robustez: Monte Carlo (barajar el orden de operaciones y meter pequeños cambios miles de veces: ¿aguanta o era suerte?) + walk-forward (repetir el ajuste avanzando en el tiempo)</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
@@ -3236,11 +3214,11 @@
         <v>1</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>04.03.02 (pendiente, Constructores)</t>
+          <t>04.03.03 (pendiente, Validador)</t>
         </is>
       </c>
     </row>
@@ -3252,12 +3230,12 @@
       </c>
       <c r="B43" s="33" t="inlineStr">
         <is>
-          <t>04.03.04</t>
+          <t>04.03.05</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Robustez: Monte Carlo (barajar el orden de operaciones y meter pequeños cambios miles de veces: ¿aguanta o era suerte?) + walk-forward (repetir el ajuste avanzando en el tiempo)</t>
+          <t>Veredicto pasa/no pasa por variante, con los criterios de G2. Quien construyó no vota</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
@@ -3279,11 +3257,11 @@
         <v>1</v>
       </c>
       <c r="H43" s="5" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>04.03.03 (pendiente, Validador)</t>
+          <t>04.03.04 (pendiente, Validador)</t>
         </is>
       </c>
     </row>
@@ -3295,17 +3273,17 @@
       </c>
       <c r="B44" s="33" t="inlineStr">
         <is>
-          <t>04.03.05</t>
+          <t>04.04.01</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Veredicto pasa/no pasa por variante, con los criterios de G2. Quien construyó no vota</t>
+          <t>Informe de la vuelta: qué pasó, qué murió y por qué. Registro de TODAS las pruebas, también fallidas</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Validador</t>
+          <t>Secretario</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -3319,14 +3297,14 @@
         </is>
       </c>
       <c r="G44" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H44" s="5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>04.03.04 (pendiente, Validador)</t>
+          <t>04.03.05 (pendiente, Validador)</t>
         </is>
       </c>
     </row>
@@ -3338,17 +3316,17 @@
       </c>
       <c r="B45" s="33" t="inlineStr">
         <is>
-          <t>04.04.01</t>
+          <t>04.04.02</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Informe de la vuelta: qué pasó, qué murió y por qué. Registro de TODAS las pruebas, también fallidas</t>
+          <t>Si ninguna pasa: volver a 04.02 con lecciones (vuelta 2, 3…). Tras la 3ª vuelta sin éxito: revisión completa del planteamiento con el CEO</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Secretario</t>
+          <t>Orquestador</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -3361,15 +3339,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="G45" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="H45" s="5" t="n">
-        <v>7</v>
-      </c>
+      <c r="G45" s="5" t="inlineStr"/>
+      <c r="H45" s="5" t="inlineStr"/>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>04.03.05 (pendiente, Validador)</t>
+          <t>04.04.01 (pendiente, Secretario)</t>
         </is>
       </c>
     </row>
@@ -3381,17 +3355,17 @@
       </c>
       <c r="B46" s="33" t="inlineStr">
         <is>
-          <t>04.04.02</t>
+          <t>04.04.03</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Si ninguna pasa: volver a 04.02 con lecciones (vuelta 2, 3…). Tras la 3ª vuelta sin éxito: revisión completa del planteamiento con el CEO</t>
-        </is>
-      </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>Orquestador</t>
+          <t>PUERTA G2: el CEO decide qué pasa a demo</t>
+        </is>
+      </c>
+      <c r="D46" s="28" t="inlineStr">
+        <is>
+          <t>CEO</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -3404,8 +3378,12 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="G46" s="5" t="inlineStr"/>
-      <c r="H46" s="5" t="inlineStr"/>
+      <c r="G46" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H46" s="5" t="n">
+        <v>5</v>
+      </c>
       <c r="I46" s="4" t="inlineStr">
         <is>
           <t>04.04.01 (pendiente, Secretario)</t>
@@ -3420,17 +3398,17 @@
       </c>
       <c r="B47" s="33" t="inlineStr">
         <is>
-          <t>04.04.03</t>
+          <t>05.01.01</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>PUERTA G2: el CEO decide qué pasa a demo</t>
-        </is>
-      </c>
-      <c r="D47" s="28" t="inlineStr">
-        <is>
-          <t>CEO</t>
+          <t>Bot en demo, solo y con guardias automáticos</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>Constructores</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -3447,11 +3425,11 @@
         <v>1</v>
       </c>
       <c r="H47" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I47" s="4" t="inlineStr">
         <is>
-          <t>04.04.01 (pendiente, Secretario)</t>
+          <t>04.04.03 (pendiente, CEO)</t>
         </is>
       </c>
     </row>
@@ -3463,17 +3441,17 @@
       </c>
       <c r="B48" s="33" t="inlineStr">
         <is>
-          <t>05.01.01</t>
+          <t>05.01.02</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Bot en demo, solo y con guardias automáticos</t>
+          <t>Seguimiento semanal real vs. prometido (8-12 semanas)</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Constructores</t>
+          <t>Secretario</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -3490,11 +3468,11 @@
         <v>1</v>
       </c>
       <c r="H48" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I48" s="4" t="inlineStr">
         <is>
-          <t>04.04.03 (pendiente, CEO)</t>
+          <t>05.01.01 (pendiente, Constructores)</t>
         </is>
       </c>
     </row>
@@ -3506,17 +3484,17 @@
       </c>
       <c r="B49" s="33" t="inlineStr">
         <is>
-          <t>05.01.02</t>
+          <t>05.01.03</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Seguimiento semanal real vs. prometido (8-12 semanas)</t>
-        </is>
-      </c>
-      <c r="D49" s="4" t="inlineStr">
-        <is>
-          <t>Secretario</t>
+          <t>PUERTA G3: CEO decide dinero, cuánto y pérdida máxima</t>
+        </is>
+      </c>
+      <c r="D49" s="28" t="inlineStr">
+        <is>
+          <t>CEO</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -3533,11 +3511,11 @@
         <v>1</v>
       </c>
       <c r="H49" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I49" s="4" t="inlineStr">
         <is>
-          <t>05.01.01 (pendiente, Constructores)</t>
+          <t>05.01.02 (pendiente, Secretario)</t>
         </is>
       </c>
     </row>
@@ -3549,17 +3527,17 @@
       </c>
       <c r="B50" s="33" t="inlineStr">
         <is>
-          <t>05.01.03</t>
+          <t>06.01.01</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>PUERTA G3: CEO decide dinero, cuánto y pérdida máxima</t>
-        </is>
-      </c>
-      <c r="D50" s="28" t="inlineStr">
-        <is>
-          <t>CEO</t>
+          <t>Dinero pequeño respetando los límites de 01.01.03</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>Constructores</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -3576,11 +3554,11 @@
         <v>1</v>
       </c>
       <c r="H50" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I50" s="4" t="inlineStr">
         <is>
-          <t>05.01.02 (pendiente, Secretario)</t>
+          <t>05.01.03 (pendiente, CEO)</t>
         </is>
       </c>
     </row>
@@ -3592,17 +3570,17 @@
       </c>
       <c r="B51" s="33" t="inlineStr">
         <is>
-          <t>06.01.01</t>
+          <t>06.01.02</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Dinero pequeño respetando los límites de 01.01.03</t>
-        </is>
-      </c>
-      <c r="D51" s="4" t="inlineStr">
-        <is>
-          <t>Constructores</t>
+          <t>PUERTA G4 mensual: seguir, ampliar o parar. Si pierde más de lo escrito, se para sin discusión</t>
+        </is>
+      </c>
+      <c r="D51" s="28" t="inlineStr">
+        <is>
+          <t>CEO</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -3615,59 +3593,16 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="G51" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H51" s="5" t="n">
-        <v>1</v>
-      </c>
+      <c r="G51" s="5" t="inlineStr"/>
+      <c r="H51" s="5" t="inlineStr"/>
       <c r="I51" s="4" t="inlineStr">
         <is>
-          <t>05.01.03 (pendiente, CEO)</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B52" s="33" t="inlineStr">
-        <is>
-          <t>06.01.02</t>
-        </is>
-      </c>
-      <c r="C52" s="4" t="inlineStr">
-        <is>
-          <t>PUERTA G4 mensual: seguir, ampliar o parar. Si pierde más de lo escrito, se para sin discusión</t>
-        </is>
-      </c>
-      <c r="D52" s="28" t="inlineStr">
-        <is>
-          <t>CEO</t>
-        </is>
-      </c>
-      <c r="E52" s="5" t="inlineStr">
-        <is>
-          <t>PRODUCTO</t>
-        </is>
-      </c>
-      <c r="F52" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G52" s="5" t="inlineStr"/>
-      <c r="H52" s="5" t="inlineStr"/>
-      <c r="I52" s="4" t="inlineStr">
-        <is>
           <t>06.01.01 (pendiente, Constructores)</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="46" customHeight="1">
-      <c r="A54" s="35" t="inlineStr">
+    <row r="53" ht="46" customHeight="1">
+      <c r="A53" s="35" t="inlineStr">
         <is>
           <t>Aviso de la regla 8 (CLAUDE.md): si la cola de arriba solo tuviera tareas de MOTOR, hay que parar y avisar al CEO; significa que la cola esta mal llena. Ahora mismo la cola tiene 5 de producto y 12 de motor.</t>
         </is>
@@ -3684,8 +3619,8 @@
     <mergeCell ref="A9:I9"/>
     <mergeCell ref="A27:I27"/>
     <mergeCell ref="C4:H4"/>
+    <mergeCell ref="A53:I53"/>
     <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A54:I54"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4307,15 +4242,15 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>En curso</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr"/>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>FICHA SEGUNDA PASADA (02/08): PUNTO DE PARTIDA: la primera pasada dio RECHAZA el 31/07 con 7 motivos, y ese veredicto solo existe dentro de esta celda del WBS: no hay artefacto en disco. Entremedias el CEO aprobó los siete criterios de G1 en D-11 (00-direccion/DECISIONES.md), que dice resolver parte de esos motivos. ALCANCE — un veredicto por cada uno de los 7 motivos, con la etiqueta CERRADO o ABIERTO y la prueba al lado: (1) Dos criterios de G1 sin dato («cientos de operaciones posibles» y […] texto completo en 00-direccion/WBS.md</t>
-        </is>
-      </c>
+          <t>Hecha</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>02/08 — 04-resultados/veredictos/veredicto_fase_02.md y 03-motor/scripts/deriva_oro.py. Segunda pasada del RECHAZA del 31/07. ACEPTA CON HUECOS DECLARADOS, válido SOLO si el defecto del motivo 5 llega declarado al CEO en la ficha de G1; si se omite, decae y rige el RECHAZA. Balance: 4 cerrados (1, 3, 6, 7), 3 abiertos (2, 4, 5), el 5 escalado. Motivo 3 zanjado por ejecución: XAUUSD a 4h pasa de 2,32% a 4,22% y 5,43%, bajo el umbral del 10%, así que la deriva del coste del oro NO cambia el veredicto a 4h; sí lo rompe a 1h (11,01%) y a 15m (19,80-25,46%). Motivo 5 confirmado uno a uno: 7 de 8 instrumentos** mezclan broker o tipo de cuenta; solo BTCUSD comparte fuente. RECORRIDO: validador […] texto completo en 00-direccion/WBS.md</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="13" t="inlineStr">

</xml_diff>

<commit_message>
03.01.18: contador producto/motor + regla 8 reactivada
Contador en .claude/hooks/contador_producto_motor.py, montado como hook
SessionStart en .claude/settings.json.

CRITERIO DE HECHO CUMPLIDO: sobre los 16 commits de referencia del 01/08
(da1e3c7..79902cb) da 7 motor / 9 producto / 0 papeleo = 43,8%, el mismo
numero que la clasificacion manual por contenido de INFORME_AWESOME.md.

Clasifica TODOS los commits, no solo los que llevan codigo WBS: esa era la
ceguera que dio 20,0% cuando el real era 43,8% (L-016). El fichero no tiene
ninguna rama que filtre por codigo WBS antes de contar.
03-motor/** no se usa nunca como criterio: esa carpeta contiene producto.

Regla 8 reactivada en CLAUDE.md. El reparto medido hoy al reactivarla es del
58,9% de motor sobre 58 commits, casi el triple del techo.

settings.json: cambio SOLO aditivo. Las 10 reglas deny y la lista allow
quedan byte a byte iguales, comprobado contra HEAD.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/05-vista-ceo/WBS_Bot_Trading_v0.9.xlsx
+++ b/05-vista-ceo/WBS_Bot_Trading_v0.9.xlsx
@@ -1428,7 +1428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1527,7 +1527,7 @@
       <c r="B6" s="30" t="n"/>
       <c r="C6" s="31" t="inlineStr">
         <is>
-          <t>04.02.01 — Barrido de fuentes: papers, libros, foros, GitHub, X. Regla: mínimo 2 fuentes independientes verificables por idea; vendedores de cursos/señales no son fuente. Detras de ella esperan 16 de las 37 tareas vivas.</t>
+          <t>04.02.01 — Barrido de fuentes: papers, libros, foros, GitHub, X. Regla: mínimo 2 fuentes independientes verificables por idea; vendedores de cursos/señales no son fuente. Detras de ella esperan 16 de las 36 tareas vivas.</t>
         </is>
       </c>
       <c r="D6" s="30" t="n"/>
@@ -1591,7 +1591,7 @@
     <row r="9">
       <c r="A9" s="32" t="inlineStr">
         <is>
-          <t>SE PUEDE TRABAJAR YA — 16 tareas, en este orden</t>
+          <t>SE PUEDE TRABAJAR YA — 15 tareas, en este orden</t>
         </is>
       </c>
       <c r="B9" s="32" t="n"/>
@@ -2114,12 +2114,12 @@
       </c>
       <c r="B23" s="33" t="inlineStr">
         <is>
-          <t>03.01.18</t>
+          <t>07.01.01</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>NUEVA 03/08 (D-20, idea 1 de las auditorías): contador mecánico del reparto producto/motor, inyectado en el contexto al arrancar cada tirada</t>
+          <t>Carpetas y documentos en orden; una fuente de verdad por tema; lo sustituido se borra</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -2151,12 +2151,12 @@
       </c>
       <c r="B24" s="33" t="inlineStr">
         <is>
-          <t>07.01.01</t>
+          <t>07.01.02</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Carpetas y documentos en orden; una fuente de verdad por tema; lo sustituido se borra</t>
+          <t>Mejoras del motor: SOLO tareas aprobadas en revisión semanal (el motor no manda)</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -2183,56 +2183,58 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="n">
-        <v>16</v>
-      </c>
-      <c r="B25" s="33" t="inlineStr">
-        <is>
-          <t>07.01.02</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>Mejoras del motor: SOLO tareas aprobadas en revisión semanal (el motor no manda)</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>Constructores</t>
-        </is>
-      </c>
-      <c r="E25" s="34" t="inlineStr">
+      <c r="A25" s="32" t="inlineStr">
+        <is>
+          <t>ESPERANDO A OTRA TAREA — 21 tareas, en orden de codigo WBS</t>
+        </is>
+      </c>
+      <c r="B25" s="32" t="n"/>
+      <c r="C25" s="32" t="n"/>
+      <c r="D25" s="32" t="n"/>
+      <c r="E25" s="32" t="n"/>
+      <c r="F25" s="32" t="n"/>
+      <c r="G25" s="32" t="n"/>
+      <c r="H25" s="32" t="n"/>
+      <c r="I25" s="32" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B26" s="33" t="inlineStr">
+        <is>
+          <t>03.01.05</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>PRUEBA REAL DEL MOTOR: un día entero de trabajo desatendido de verdad antes de dar la fase por buena</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Orquestador</t>
+        </is>
+      </c>
+      <c r="E26" s="34" t="inlineStr">
         <is>
           <t>MOTOR</t>
         </is>
       </c>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="F26" s="5" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr"/>
-      <c r="H25" s="5" t="inlineStr"/>
-      <c r="I25" s="4" t="inlineStr">
-        <is>
-          <t>nada: se puede empezar ya</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="32" t="inlineStr">
-        <is>
-          <t>ESPERANDO A OTRA TAREA — 21 tareas, en orden de codigo WBS</t>
-        </is>
-      </c>
-      <c r="B26" s="32" t="n"/>
-      <c r="C26" s="32" t="n"/>
-      <c r="D26" s="32" t="n"/>
-      <c r="E26" s="32" t="n"/>
-      <c r="F26" s="32" t="n"/>
-      <c r="G26" s="32" t="n"/>
-      <c r="H26" s="32" t="n"/>
-      <c r="I26" s="32" t="n"/>
+      <c r="G26" s="5" t="inlineStr"/>
+      <c r="H26" s="5" t="inlineStr"/>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
+          <t>03.01.03 (pendiente, Constructores), 03.01.04 (pendiente, Constructores)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -2242,17 +2244,17 @@
       </c>
       <c r="B27" s="33" t="inlineStr">
         <is>
-          <t>03.01.05</t>
+          <t>03.01.07</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>PRUEBA REAL DEL MOTOR: un día entero de trabajo desatendido de verdad antes de dar la fase por buena</t>
+          <t>Cola de aprobación del CEO: tabla con desplegable Aprobado / Saltar / Corregir y columna de corrección. Lo aprobado se ejecuta solo; lo corregido se rehace Y la corrección se guarda en LECCIONES.md</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Orquestador</t>
+          <t>Secretario</t>
         </is>
       </c>
       <c r="E27" s="34" t="inlineStr">
@@ -2269,7 +2271,7 @@
       <c r="H27" s="5" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>03.01.03 (pendiente, Constructores), 03.01.04 (pendiente, Constructores)</t>
+          <t>03.01.06 (pendiente, Secretario)</t>
         </is>
       </c>
     </row>
@@ -2281,17 +2283,17 @@
       </c>
       <c r="B28" s="33" t="inlineStr">
         <is>
-          <t>03.01.07</t>
+          <t>03.01.11</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Cola de aprobación del CEO: tabla con desplegable Aprobado / Saltar / Corregir y columna de corrección. Lo aprobado se ejecuta solo; lo corregido se rehace Y la corrección se guarda en LECCIONES.md</t>
+          <t>NUEVA 31/07 (D-10): guardia del cajon reservado por cifrado. Script cajon_reservado.py: la contraseña solo la tiene el CEO, no se guarda, se pide en cada operacion y nada se descifra a disco</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Secretario</t>
+          <t>Constructores</t>
         </is>
       </c>
       <c r="E28" s="34" t="inlineStr">
@@ -2299,16 +2301,16 @@
           <t>MOTOR</t>
         </is>
       </c>
-      <c r="F28" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="F28" s="14" t="inlineStr">
+        <is>
+          <t>En curso</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr"/>
       <c r="H28" s="5" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>03.01.06 (pendiente, Secretario)</t>
+          <t>03.01.08 (en curso, Crítico)</t>
         </is>
       </c>
     </row>
@@ -2320,34 +2322,34 @@
       </c>
       <c r="B29" s="33" t="inlineStr">
         <is>
-          <t>03.01.11</t>
+          <t>04.01.02</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>NUEVA 31/07 (D-10): guardia del cajon reservado por cifrado. Script cajon_reservado.py: la contraseña solo la tiene el CEO, no se guarda, se pide en cada operacion y nada se descifra a disco</t>
+          <t>Recalcular costes con precios reales del broker (sustituye 02.01.02) REQUISITO AÑADIDO 04/08: al recalcular con precios reales se comprueba que la entidad que publica la tarifa es la misma con la que se opera. Si no coinciden, la cifra vieja no se hereda: se vuelve a medir.</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Constructores</t>
-        </is>
-      </c>
-      <c r="E29" s="34" t="inlineStr">
-        <is>
-          <t>MOTOR</t>
-        </is>
-      </c>
-      <c r="F29" s="14" t="inlineStr">
-        <is>
-          <t>En curso</t>
+          <t>Constructor datos</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>PRODUCTO</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr"/>
       <c r="H29" s="5" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>03.01.08 (en curso, Crítico)</t>
+          <t>04.01.01 (en curso, CEO + Orquestador)</t>
         </is>
       </c>
     </row>
@@ -2359,12 +2361,12 @@
       </c>
       <c r="B30" s="33" t="inlineStr">
         <is>
-          <t>04.01.02</t>
+          <t>04.01.03</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Recalcular costes con precios reales del broker (sustituye 02.01.02) REQUISITO AÑADIDO 04/08: al recalcular con precios reales se comprueba que la entidad que publica la tarifa es la misma con la que se opera. Si no coinciden, la cifra vieja no se hereda: se vuelve a medir.</t>
+          <t>Histórico limpio partido en 3 cajones: construir (train), ajustar (validación) y RESERVADO bajo llave (OOS, se abre una sola vez por variante). Ningún agente toca el reservado</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
@@ -2382,8 +2384,12 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="G30" s="5" t="inlineStr"/>
-      <c r="H30" s="5" t="inlineStr"/>
+      <c r="G30" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H30" s="5" t="n">
+        <v>13</v>
+      </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
           <t>04.01.01 (en curso, CEO + Orquestador)</t>
@@ -2398,17 +2404,17 @@
       </c>
       <c r="B31" s="33" t="inlineStr">
         <is>
-          <t>04.01.03</t>
+          <t>04.02.02</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Histórico limpio partido en 3 cajones: construir (train), ajustar (validación) y RESERVADO bajo llave (OOS, se abre una sola vez por variante). Ningún agente toca el reservado</t>
+          <t>Ficha por hipótesis: por qué existiría la ventaja, reglas de entrada/salida, mercado y vela. Sin lógica de por qué gana, no entra (nada de probar por probar)</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Constructor datos</t>
+          <t>Investigador</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -2425,11 +2431,11 @@
         <v>1</v>
       </c>
       <c r="H31" s="5" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>04.01.01 (en curso, CEO + Orquestador)</t>
+          <t>04.02.01 (pendiente, Investigador)</t>
         </is>
       </c>
     </row>
@@ -2441,17 +2447,17 @@
       </c>
       <c r="B32" s="33" t="inlineStr">
         <is>
-          <t>04.02.02</t>
+          <t>04.02.03</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Ficha por hipótesis: por qué existiría la ventaja, reglas de entrada/salida, mercado y vela. Sin lógica de por qué gana, no entra (nada de probar por probar)</t>
+          <t>Filtro de sentido: el Validador puntúa y se eligen las 3-5 mejores</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Investigador</t>
+          <t>Validador</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -2468,11 +2474,11 @@
         <v>1</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>04.02.01 (pendiente, Investigador)</t>
+          <t>04.02.02 (pendiente, Investigador)</t>
         </is>
       </c>
     </row>
@@ -2484,12 +2490,12 @@
       </c>
       <c r="B33" s="33" t="inlineStr">
         <is>
-          <t>04.02.03</t>
+          <t>04.02.04</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Filtro de sentido: el Validador puntúa y se eligen las 3-5 mejores</t>
+          <t>Pre-registro de variantes: cada hipótesis deja escritas sus variantes ANTES de probar (máx. 5-7 por hipótesis). Lo no registrado no se prueba</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
@@ -2511,11 +2517,11 @@
         <v>1</v>
       </c>
       <c r="H33" s="5" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>04.02.02 (pendiente, Investigador)</t>
+          <t>04.02.03 (pendiente, Validador)</t>
         </is>
       </c>
     </row>
@@ -2527,17 +2533,17 @@
       </c>
       <c r="B34" s="33" t="inlineStr">
         <is>
-          <t>04.02.04</t>
+          <t>04.03.01</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Pre-registro de variantes: cada hipótesis deja escritas sus variantes ANTES de probar (máx. 5-7 por hipótesis). Lo no registrado no se prueba</t>
+          <t>Backtest con costes reales sobre el cajón de construir</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Validador</t>
+          <t>Constructores</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -2554,11 +2560,11 @@
         <v>1</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>04.02.03 (pendiente, Validador)</t>
+          <t>04.01.03 (pendiente, Constructor datos), 04.02.04 (pendiente, Validador)</t>
         </is>
       </c>
     </row>
@@ -2570,12 +2576,12 @@
       </c>
       <c r="B35" s="33" t="inlineStr">
         <is>
-          <t>04.03.01</t>
+          <t>04.03.02</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Backtest con costes reales sobre el cajón de construir</t>
+          <t>Ajuste SOLO con el cajón de validación; lo que no aguanta, muere aquí</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -2597,11 +2603,11 @@
         <v>1</v>
       </c>
       <c r="H35" s="5" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>04.01.03 (pendiente, Constructor datos), 04.02.04 (pendiente, Validador)</t>
+          <t>04.03.01 (pendiente, Constructores)</t>
         </is>
       </c>
     </row>
@@ -2613,17 +2619,17 @@
       </c>
       <c r="B36" s="33" t="inlineStr">
         <is>
-          <t>04.03.02</t>
+          <t>04.03.03</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Ajuste SOLO con el cajón de validación; lo que no aguanta, muere aquí</t>
+          <t>Prueba de fuego: UNA sola pasada por variante sobre el cajón reservado (OOS). Repetir sería hacerse trampa</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Constructores</t>
+          <t>Validador</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -2640,11 +2646,11 @@
         <v>1</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>04.03.01 (pendiente, Constructores)</t>
+          <t>04.03.02 (pendiente, Constructores)</t>
         </is>
       </c>
     </row>
@@ -2656,12 +2662,12 @@
       </c>
       <c r="B37" s="33" t="inlineStr">
         <is>
-          <t>04.03.03</t>
+          <t>04.03.04</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Prueba de fuego: UNA sola pasada por variante sobre el cajón reservado (OOS). Repetir sería hacerse trampa</t>
+          <t>Robustez: Monte Carlo (barajar el orden de operaciones y meter pequeños cambios miles de veces: ¿aguanta o era suerte?) + walk-forward (repetir el ajuste avanzando en el tiempo)</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -2683,11 +2689,11 @@
         <v>1</v>
       </c>
       <c r="H37" s="5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>04.03.02 (pendiente, Constructores)</t>
+          <t>04.03.03 (pendiente, Validador)</t>
         </is>
       </c>
     </row>
@@ -2699,12 +2705,12 @@
       </c>
       <c r="B38" s="33" t="inlineStr">
         <is>
-          <t>04.03.04</t>
+          <t>04.03.05</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Robustez: Monte Carlo (barajar el orden de operaciones y meter pequeños cambios miles de veces: ¿aguanta o era suerte?) + walk-forward (repetir el ajuste avanzando en el tiempo)</t>
+          <t>Veredicto pasa/no pasa por variante, con los criterios de G2. Quien construyó no vota</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
@@ -2726,11 +2732,11 @@
         <v>1</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>04.03.03 (pendiente, Validador)</t>
+          <t>04.03.04 (pendiente, Validador)</t>
         </is>
       </c>
     </row>
@@ -2742,17 +2748,17 @@
       </c>
       <c r="B39" s="33" t="inlineStr">
         <is>
-          <t>04.03.05</t>
+          <t>04.04.01</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Veredicto pasa/no pasa por variante, con los criterios de G2. Quien construyó no vota</t>
+          <t>Informe de la vuelta: qué pasó, qué murió y por qué. Registro de TODAS las pruebas, también fallidas</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Validador</t>
+          <t>Secretario</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -2766,14 +2772,14 @@
         </is>
       </c>
       <c r="G39" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H39" s="5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>04.03.04 (pendiente, Validador)</t>
+          <t>04.03.05 (pendiente, Validador)</t>
         </is>
       </c>
     </row>
@@ -2785,17 +2791,17 @@
       </c>
       <c r="B40" s="33" t="inlineStr">
         <is>
-          <t>04.04.01</t>
+          <t>04.04.02</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Informe de la vuelta: qué pasó, qué murió y por qué. Registro de TODAS las pruebas, también fallidas</t>
+          <t>Si ninguna pasa: volver a 04.02 con lecciones (vuelta 2, 3…). Tras la 3ª vuelta sin éxito: revisión completa del planteamiento con el CEO</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Secretario</t>
+          <t>Orquestador</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -2808,15 +2814,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="G40" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="H40" s="5" t="n">
-        <v>7</v>
-      </c>
+      <c r="G40" s="5" t="inlineStr"/>
+      <c r="H40" s="5" t="inlineStr"/>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>04.03.05 (pendiente, Validador)</t>
+          <t>04.04.01 (pendiente, Secretario)</t>
         </is>
       </c>
     </row>
@@ -2828,17 +2830,17 @@
       </c>
       <c r="B41" s="33" t="inlineStr">
         <is>
-          <t>04.04.02</t>
+          <t>04.04.03</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Si ninguna pasa: volver a 04.02 con lecciones (vuelta 2, 3…). Tras la 3ª vuelta sin éxito: revisión completa del planteamiento con el CEO</t>
-        </is>
-      </c>
-      <c r="D41" s="4" t="inlineStr">
-        <is>
-          <t>Orquestador</t>
+          <t>PUERTA G2: el CEO decide qué pasa a demo</t>
+        </is>
+      </c>
+      <c r="D41" s="28" t="inlineStr">
+        <is>
+          <t>CEO</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -2851,8 +2853,12 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="G41" s="5" t="inlineStr"/>
-      <c r="H41" s="5" t="inlineStr"/>
+      <c r="G41" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H41" s="5" t="n">
+        <v>5</v>
+      </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
           <t>04.04.01 (pendiente, Secretario)</t>
@@ -2867,17 +2873,17 @@
       </c>
       <c r="B42" s="33" t="inlineStr">
         <is>
-          <t>04.04.03</t>
+          <t>05.01.01</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>PUERTA G2: el CEO decide qué pasa a demo</t>
-        </is>
-      </c>
-      <c r="D42" s="28" t="inlineStr">
-        <is>
-          <t>CEO</t>
+          <t>Bot en demo, solo y con guardias automáticos</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>Constructores</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -2894,11 +2900,11 @@
         <v>1</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>04.04.01 (pendiente, Secretario)</t>
+          <t>04.04.03 (pendiente, CEO)</t>
         </is>
       </c>
     </row>
@@ -2910,17 +2916,17 @@
       </c>
       <c r="B43" s="33" t="inlineStr">
         <is>
-          <t>05.01.01</t>
+          <t>05.01.02</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Bot en demo, solo y con guardias automáticos</t>
+          <t>Seguimiento semanal real vs. prometido (8-12 semanas)</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Constructores</t>
+          <t>Secretario</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -2937,11 +2943,11 @@
         <v>1</v>
       </c>
       <c r="H43" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>04.04.03 (pendiente, CEO)</t>
+          <t>05.01.01 (pendiente, Constructores)</t>
         </is>
       </c>
     </row>
@@ -2953,17 +2959,17 @@
       </c>
       <c r="B44" s="33" t="inlineStr">
         <is>
-          <t>05.01.02</t>
+          <t>05.01.03</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Seguimiento semanal real vs. prometido (8-12 semanas)</t>
-        </is>
-      </c>
-      <c r="D44" s="4" t="inlineStr">
-        <is>
-          <t>Secretario</t>
+          <t>PUERTA G3: CEO decide dinero, cuánto y pérdida máxima</t>
+        </is>
+      </c>
+      <c r="D44" s="28" t="inlineStr">
+        <is>
+          <t>CEO</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -2980,11 +2986,11 @@
         <v>1</v>
       </c>
       <c r="H44" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>05.01.01 (pendiente, Constructores)</t>
+          <t>05.01.02 (pendiente, Secretario)</t>
         </is>
       </c>
     </row>
@@ -2996,17 +3002,17 @@
       </c>
       <c r="B45" s="33" t="inlineStr">
         <is>
-          <t>05.01.03</t>
+          <t>06.01.01</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>PUERTA G3: CEO decide dinero, cuánto y pérdida máxima</t>
-        </is>
-      </c>
-      <c r="D45" s="28" t="inlineStr">
-        <is>
-          <t>CEO</t>
+          <t>Dinero pequeño respetando los límites de 01.01.03</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>Constructores</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -3023,11 +3029,11 @@
         <v>1</v>
       </c>
       <c r="H45" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>05.01.02 (pendiente, Secretario)</t>
+          <t>05.01.03 (pendiente, CEO)</t>
         </is>
       </c>
     </row>
@@ -3039,17 +3045,17 @@
       </c>
       <c r="B46" s="33" t="inlineStr">
         <is>
-          <t>06.01.01</t>
+          <t>06.01.02</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Dinero pequeño respetando los límites de 01.01.03</t>
-        </is>
-      </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>Constructores</t>
+          <t>PUERTA G4 mensual: seguir, ampliar o parar. Si pierde más de lo escrito, se para sin discusión</t>
+        </is>
+      </c>
+      <c r="D46" s="28" t="inlineStr">
+        <is>
+          <t>CEO</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -3062,76 +3068,33 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="G46" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H46" s="5" t="n">
-        <v>1</v>
-      </c>
+      <c r="G46" s="5" t="inlineStr"/>
+      <c r="H46" s="5" t="inlineStr"/>
       <c r="I46" s="4" t="inlineStr">
         <is>
-          <t>05.01.03 (pendiente, CEO)</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B47" s="33" t="inlineStr">
-        <is>
-          <t>06.01.02</t>
-        </is>
-      </c>
-      <c r="C47" s="4" t="inlineStr">
-        <is>
-          <t>PUERTA G4 mensual: seguir, ampliar o parar. Si pierde más de lo escrito, se para sin discusión</t>
-        </is>
-      </c>
-      <c r="D47" s="28" t="inlineStr">
-        <is>
-          <t>CEO</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr">
-        <is>
-          <t>PRODUCTO</t>
-        </is>
-      </c>
-      <c r="F47" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G47" s="5" t="inlineStr"/>
-      <c r="H47" s="5" t="inlineStr"/>
-      <c r="I47" s="4" t="inlineStr">
-        <is>
           <t>06.01.01 (pendiente, Constructores)</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="46" customHeight="1">
-      <c r="A49" s="35" t="inlineStr">
-        <is>
-          <t>Aviso de la regla 8 (CLAUDE.md): si la cola de arriba solo tuviera tareas de MOTOR, hay que parar y avisar al CEO; significa que la cola esta mal llena. Ahora mismo la cola tiene 3 de producto y 13 de motor.</t>
+    <row r="48" ht="46" customHeight="1">
+      <c r="A48" s="35" t="inlineStr">
+        <is>
+          <t>Aviso de la regla 8 (CLAUDE.md): si la cola de arriba solo tuviera tareas de MOTOR, hay que parar y avisar al CEO; significa que la cola esta mal llena. Ahora mismo la cola tiene 3 de producto y 12 de motor.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A26:I26"/>
     <mergeCell ref="C6:H6"/>
+    <mergeCell ref="A25:I25"/>
     <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A49:I49"/>
     <mergeCell ref="C5:H5"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A9:I9"/>
     <mergeCell ref="C4:H4"/>
+    <mergeCell ref="A48:I48"/>
     <mergeCell ref="A6:B6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4353,15 +4316,15 @@
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F40" s="4" t="inlineStr"/>
-      <c r="G40" s="4" t="inlineStr">
-        <is>
-          <t>FICHA (03/08): Problema, medido y no supuesto: el techo del 20% de motor de la regla 8 de CLAUDE.md es prosa y nadie lo mide. La primera vez que se midió, el 01/08, el reparto real era 7 de 16 commits, 43,8%, más del doble del techo, y el proyecto llevaba desde el arranque sin saberlo. Qué se construye: un hook SessionStart que calcula el reparto desde git log y lo inyecta en el contexto con hookSpecificOutput.additionalContext, de forma que cada tirada empiece con el número delante en vez de […] texto completo en 00-direccion/WBS.md</t>
-        </is>
-      </c>
+          <t>Hecha</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>12/08 — contador .claude/hooks/contador_producto_motor.py, hook SessionStart montado; reproduce 43,8% sobre los 16 commits del 01/08 FICHA (03/08): Problema, medido y no supuesto: el techo del 20% de motor de la regla 8 de CLAUDE.md es prosa y nadie lo mide. La primera vez que se midió, el 01/08, el reparto real era 7 de 16 commits, 43,8%, más del doble del techo, y el proyecto llevaba desde el arranque sin saberlo. Qué se construye: un hook SessionStart que calcula el reparto desde git log y lo inyecta en el contexto con hookSpecificOutput.additionalContext, de forma que cada tirada empiece con el número delante en vez de con la buena intención. Regla de clasificación obligatoria, ya […] texto completo en 00-direccion/WBS.md</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="13" t="inlineStr">

</xml_diff>

<commit_message>
meta: D-35 y D-36 firmadas, regla 3 retirada y 10 fusionada
28 reglas en CLAUDE.md. Tabla de correspondencia vieja->nueva anadida:
las ~800 citas antiguas siguen siendo legibles y no se reescribe el pasado
(DECISIONES.md y LECCIONES.md solo admiten anadir).
Remapeadas las citas de los 14 ficheros vivos de .claude/ y del propio CLAUDE.md.
Dos citas huerfanas reales arregladas en generar_excel.py.
verificar_excel.py: 0 fallos, 9 avisos (misma base que antes).

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/05-vista-ceo/WBS_Bot_Trading_v0.9.xlsx
+++ b/05-vista-ceo/WBS_Bot_Trading_v0.9.xlsx
@@ -1328,7 +1328,7 @@
     <row r="9">
       <c r="A9" s="15" t="inlineStr">
         <is>
-          <t>FORMATO OBLIGATORIO DE FICHA DE DECISION (regla 10)</t>
+          <t>FORMATO OBLIGATORIO DE FICHA DE DECISION (seccion 'Que llega al CEO' de CLAUDE.md)</t>
         </is>
       </c>
     </row>
@@ -6258,7 +6258,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -6268,7 +6268,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>LAS 30 REGLAS — mandan sobre cualquier otra instruccion</t>
+          <t>LAS 28 REGLAS — mandan sobre cualquier otra instruccion</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -6319,7 +6319,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Los códigos son estables: una tarea empezada no se renumera jamás.</t>
+          <t>Se va en orden salvo las marcadas paralelas. Una tarea no se cierra sin cumplir su criterio de "hecho".</t>
         </is>
       </c>
     </row>
@@ -6329,7 +6329,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Se va en orden salvo las marcadas paralelas. Una tarea no se cierra sin cumplir su criterio de "hecho".</t>
+          <t>La ficha de una tarea se escribe en la cola ANTES de trabajarla, nunca al cerrarla. Sin ficha, no hay tarea.</t>
         </is>
       </c>
     </row>
@@ -6339,7 +6339,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>La ficha de una tarea se escribe en la cola ANTES de trabajarla, nunca al cerrarla. Sin ficha, no hay tarea.</t>
+          <t>Regla de no-ambigüedad: toda tarea debe poder ejecutarse sin adivinar nada. Si tienes que suponer algo, devuelve la tarea al orquestador para que la reescriba. No supongas.</t>
         </is>
       </c>
     </row>
@@ -6349,245 +6349,225 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Regla de no-ambigüedad: toda tarea debe poder ejecutarse sin adivinar nada. Si tienes que suponer algo, devuelve la tarea al orquestador para que la reescriba. No supongas.</t>
+          <t>Ningún criterio de hecho exige una herramienta que el ejecutor no tiene. Antes de escribirlo, se localiza por grep la línea tools: del agente que va a ejecutarlo. Si la prueba exige algo que no aparece ahí, la prueba se traslada al revisor. Un agente al que se le pide lo imposible no falla: fabrica, y el fallo se le acaba imputando a él en vez de a quien repartió. (D-34, 10/08/2026.)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
-        <v>30</v>
+        <v>7</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Ningún criterio de hecho exige una herramienta que el ejecutor no tiene. Antes de escribirlo, se localiza por grep la línea tools: del agente que va a ejecutarlo. Si la prueba exige algo que no aparece ahí, la prueba se traslada al revisor. Un agente al que se le pide lo imposible no falla: fabrica, y el fallo se le acaba imputando a él en vez de a quien repartió. (D-34, 10/08/2026.)</t>
+          <t>Cada tirada autónoma cierra al menos una tarea que avanza el PRODUCTO. La infraestructura que no desbloquee mecánicamente una tarea de producto se registra como deuda y no se ejecuta sin permiso del CEO.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Cada tirada autónoma cierra al menos una tarea que avanza el PRODUCTO. La infraestructura que no desbloquee mecánicamente una tarea de producto se registra como deuda y no se ejecuta sin permiso del CEO.</t>
+          <t>El trabajo de motor y orden tiene un techo del 20% del esfuerzo semanal. Si en una tirada solo hay tareas de motor disponibles, para y avisa: es señal de que la cola está mal llena.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>El trabajo de motor y orden tiene un techo del 20% del esfuerzo semanal. Si en una tirada solo hay tareas de motor disponibles, para y avisa: es señal de que la cola está mal llena.</t>
+          <t>Jerarquía de la prueba. Ninguna afirmación se acepta por consenso entre agentes:</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Jerarquía de la prueba. Ninguna afirmación se acepta por consenso entre agentes:</t>
+          <t>Un fallo reportado por un agente no es un fallo verificado. Antes de encolar o reparar: lee el componente y reproduce el fallo.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Quien discrepa aporta el experimento que zanjaría la discusión, no otro argumento. Si no hay experimento posible, sube al CEO marcado como no probado.</t>
+          <t>Ninguna referencia a una decisión entra en código o informe sin un grep previo que la localice por fichero y línea. Solo se cita lo firmado y guardado, nunca en pasado ni antes de existir.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Un fallo reportado por un agente no es un fallo verificado. Antes de encolar o reparar: lee el componente y reproduce el fallo.</t>
+          <t>Se referencia por nombre de símbolo, nunca por número de línea.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Ninguna referencia a una decisión entra en código o informe sin un grep previo que la localice por fichero y línea. Solo se cita lo firmado y guardado, nunca en pasado ni antes de existir.</t>
+          <t>Todo dato numérico se calcula sobre datos brutos, salvo que exista una fuente primaria homogénea demostrable.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Se referencia por nombre de símbolo, nunca por número de línea.</t>
+          <t>Quien implementa ejecuta y lee su artefacto completo antes de entregar. Las puertas confirman, no descubren.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Todo dato numérico se calcula sobre datos brutos, salvo que exista una fuente primaria homogénea demostrable.</t>
+          <t>Nadie valida su propio trabajo. Quien construye no revisa; quien produce las métricas no firma el veredicto.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Quien implementa ejecuta y lee su artefacto completo antes de entregar. Las puertas confirman, no descubren.</t>
+          <t>Éxito = código fiel a la especificación, NO estrategia rentable. Un backtest con mal resultado y código correcto es un éxito registrable.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Nadie valida su propio trabajo. Quien construye no revisa; quien produce las métricas no firma el veredicto.</t>
+          <t>Test de compuerta: si la justificación de un cambio no se sostiene sin citar métricas de resultado, se deniega.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Éxito = código fiel a la especificación, NO estrategia rentable. Un backtest con mal resultado y código correcto es un éxito registrable.</t>
+          <t>Pre-registro: ninguna variante se prueba sin estar registrada antes (máx. 5-7 por hipótesis). Lo no registrado no se prueba.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Test de compuerta: si la justificación de un cambio no se sostiene sin citar métricas de resultado, se deniega.</t>
+          <t>Se guardan TODAS las pruebas, también las fallidas. Saber cuántas cosas se probaron es lo que permite juzgar si la ganadora es real o casualidad.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Pre-registro: ninguna variante se prueba sin estar registrada antes (máx. 5-7 por hipótesis). Lo no registrado no se prueba.</t>
+          <t>Registros que solo permiten añadir: 04-resultados/registro-pruebas.md y 00-direccion/DECISIONES.md nunca se reescriben. Una corrección es una entrada nueva.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Se guardan TODAS las pruebas, también las fallidas. Saber cuántas cosas se probaron es lo que permite juzgar si la ganadora es real o casualidad.</t>
+          <t>El cajón 02-datos/reservado/ no se abre. Solo el CEO puede autorizar su uso, una vez por variante. Ningún agente, ningún debate, ninguna urgencia.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Registros que solo permiten añadir: 04-resultados/registro-pruebas.md y 00-direccion/DECISIONES.md nunca se reescriben. Una corrección es una entrada nueva.</t>
+          <t>Dos niveles. Lo REVERSIBLE (archivos, código, pruebas) tiene permisos amplios: git lo deshace. Lo IRREVERSIBLE (dinero real, órdenes al broker, borrar el cajón reservado, gastar dinero nuevo) lleva barrera desde el minuto uno.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>El cajón 02-datos/reservado/ no se abre. Solo el CEO puede autorizar su uso, una vez por variante. Ningún agente, ningún debate, ninguna urgencia.</t>
+          <t>Una restricción solo se añade tras un incidente real, anotada junto al incidente, y se revisa cada mes. La que no tenga incidente vivo detrás, se quita.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Dos niveles. Lo REVERSIBLE (archivos, código, pruebas) tiene permisos amplios: git lo deshace. Lo IRREVERSIBLE (dinero real, órdenes al broker, borrar el cajón reservado, gastar dinero nuevo) lleva barrera desde el minuto uno.</t>
+          <t>Toda barrera se verifica por ejecución —inyectando el caso prohibido— antes de documentarla como activa. Sin prueba: "no verificada". Un guardia presente en el código no es un guardia probado.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Una restricción solo se añade tras un incidente real, anotada junto al incidente, y se revisa cada mes. La que no tenga incidente vivo detrás, se quita.</t>
+          <t>Los guardias bloquean por defecto. La condición que activa una exención debe ser un hecho impuesto por el sistema, nunca un dato que elija el vigilado.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Toda barrera se verifica por ejecución —inyectando el caso prohibido— antes de documentarla como activa. Sin prueba: "no verificada". Un guardia presente en el código no es un guardia probado.</t>
+          <t>Los datos nunca entran en git. Se descargan con script. Comprobar el día 1 que .gitignore funciona de verdad.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Los guardias bloquean por defecto. La condición que activa una exención debe ser un hecho impuesto por el sistema, nunca un dato que elija el vigilado.</t>
+          <t>Una sola fuente de verdad por tema. Documento que se sustituye, se borra: git guarda el historial.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>Los datos nunca entran en git. Se descargan con script. Comprobar el día 1 que .gitignore funciona de verdad.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="5" t="n">
-        <v>28</v>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>Una sola fuente de verdad por tema. Documento que se sustituye, se borra: git guarda el historial.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="5" t="n">
-        <v>29</v>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>Cada agente lleva el identificador exacto de su modelo, nunca un alias, y ningún agente sin modelo.</t>
         </is>
@@ -6608,7 +6588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6620,7 +6600,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>REGISTRO DE DECISIONES (30) — solo se añade, nunca se reescribe (regla 21 de CLAUDE.md)</t>
+          <t>REGISTRO DE DECISIONES (32) — solo se añade, nunca se reescribe (regla 21 de CLAUDE.md)</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -7410,6 +7390,56 @@
 Qué significa. Ningún criterio de hecho puede exigir una comprobación que las herramientas declaradas en la línea tools: del agente que lo ejecuta no le permitan hacer. Antes de escribir un criterio de hecho se localiza esa línea por grep; si la prueba exige algo que no aparece en ella, la prueba se traslada al revisor, que sí la tiene. Queda escrito como regla 30 de CLAUDE.md.
 Qué NO hace. No cambia la línea tools: de ningún agente. En particular, secretario sigue sin Bash.
 Por qué ésta y no repartir herramientas. Del diagnóstico de 03.01.15 en 04-resultados/diagnostico_03.01.15_herramientas_agentes.md, con los ocho agentes barridos: los fallos medidos son de dos clases y solo una la arregla una herramienta. Un agente sin Bash declaró una cifra […] texto completo en 00-direccion/DECISIONES.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>D-35</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Las reglas sin incidente detrás: se retira la 3, la 10 se fusiona en la 9, quedan 28</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Qué se decide. Opción A de la ficha del apartado 3 de 00-direccion/INFORME-CIRUGIA-MOTOR.md. Palabras literales del CEO, 12/08/2026: «Retirar la regla 3. Fusionar la 10 con la 9. Dejar la 17, la 18, la 19 y la 20.»
+Motivo que el CEO ordena escribir, literal: las cuatro reglas de estrategia no tienen incidente detrás porque la fase 04 nunca ha empezado. Eso no es peso muerto: es la prueba de que el producto no ha arrancado. Retirarlas sería quitar el airbag por no haber chocado.
+Qué cambia en el disco.
+1. Vieja regla 3 («los códigos son estables: una tarea empezada no se renumera jamás») — RETIRADA. No tenía incidente detrás ni en este proyecto ni en el anterior.
+2. Vieja regla 10 («quien discrepa aporta el experimento que zanjaría la discusión») — FUSIONADA dentro de la 9, la jerarquía de la prueba, cuyo nivel 1 ya decía lo mismo. El texto no se pierde: sigue entero dentro de la regla […] texto completo en 00-direccion/DECISIONES.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>D-36</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Se aplican las barreras (a), (b) y (d) de D-29; la (c), la de gasto, se cierra por imposible</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Qué se decide. Palabras literales del CEO, 12/08/2026: «se autorizan (a), (b) y (d). El punto (c) se cierra por imposible.» Los cuatro puntos son los de 00-direccion/informes/FICHA_D-29.md.
+POR QUÉ ESTA ENTRADA EXISTE SI D-29 YA ESTABA FIRMADA, y conviene que quede claro. D-29 de este mismo fichero ya firmó las cuatro barreras el 09/08/2026 (opción A). Lo que dejó sin firmar fue el cómo: su propio texto dice que aplicar el parche de (a) y (b) a .claude/settings.json «necesita una letra aparte del CEO, porque bajo bypassPermissions (D-27) escribir ese fichero no dispara ninguna aprobación y el sistema no le preguntaría». D-36 es esa letra aparte. No repite D-29: la ejecuta.
+(a) El agujero del cajón reservado — SE AUTORIZA APLICAR. El patrón Bash( 02-datos/reservado) de .claude/settings.json exige un espacio literal y no cubre la ruta pegada a una comilla. Medido el 05/08. Se sustituye […] texto completo en 00-direccion/DECISIONES.md</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
meta: descongelar 03.01.24 y 03.01.25, autorizadas por D-36
Filas recortadas y pegadas integras desde DEUDA-MOTOR.md al WBS: verificado
byte a byte contra HEAD anterior, identicas salvo la coletilla de deuda,
sustituida por la referencia a D-36. Las otras tres filas siguen congeladas.
Metrica L-027: 64 filas de tarea, 0 rotas. verificar_excel.py: 0 fallos.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/05-vista-ceo/WBS_Bot_Trading_v0.9.xlsx
+++ b/05-vista-ceo/WBS_Bot_Trading_v0.9.xlsx
@@ -20,7 +20,7 @@
     <sheet name="LIMITES CEO" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'TAREAS'!$A$4:$G$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'TAREAS'!$A$4:$G$79</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -742,23 +742,23 @@
         </is>
       </c>
       <c r="B4" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"01.??.??")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"01.??.??")</f>
         <v/>
       </c>
       <c r="C4" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"01.??.??",TAREAS!$E$5:$E$77,"Hecha")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"01.??.??",TAREAS!$E$5:$E$79,"Hecha")</f>
         <v/>
       </c>
       <c r="D4" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"01.??.??",TAREAS!$E$5:$E$77,"En curso")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"01.??.??",TAREAS!$E$5:$E$79,"En curso")</f>
         <v/>
       </c>
       <c r="E4" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"01.??.??",TAREAS!$E$5:$E$77,"Pendiente")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"01.??.??",TAREAS!$E$5:$E$79,"Pendiente")</f>
         <v/>
       </c>
       <c r="F4" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"01.??.??",TAREAS!$E$5:$E$77,"Bloqueada")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"01.??.??",TAREAS!$E$5:$E$79,"Bloqueada")</f>
         <v/>
       </c>
       <c r="G4" s="6">
@@ -773,23 +773,23 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"02.??.??")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"02.??.??")</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"02.??.??",TAREAS!$E$5:$E$77,"Hecha")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"02.??.??",TAREAS!$E$5:$E$79,"Hecha")</f>
         <v/>
       </c>
       <c r="D5" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"02.??.??",TAREAS!$E$5:$E$77,"En curso")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"02.??.??",TAREAS!$E$5:$E$79,"En curso")</f>
         <v/>
       </c>
       <c r="E5" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"02.??.??",TAREAS!$E$5:$E$77,"Pendiente")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"02.??.??",TAREAS!$E$5:$E$79,"Pendiente")</f>
         <v/>
       </c>
       <c r="F5" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"02.??.??",TAREAS!$E$5:$E$77,"Bloqueada")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"02.??.??",TAREAS!$E$5:$E$79,"Bloqueada")</f>
         <v/>
       </c>
       <c r="G5" s="6">
@@ -804,23 +804,23 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"03.??.??")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"03.??.??")</f>
         <v/>
       </c>
       <c r="C6" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"03.??.??",TAREAS!$E$5:$E$77,"Hecha")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"03.??.??",TAREAS!$E$5:$E$79,"Hecha")</f>
         <v/>
       </c>
       <c r="D6" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"03.??.??",TAREAS!$E$5:$E$77,"En curso")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"03.??.??",TAREAS!$E$5:$E$79,"En curso")</f>
         <v/>
       </c>
       <c r="E6" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"03.??.??",TAREAS!$E$5:$E$77,"Pendiente")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"03.??.??",TAREAS!$E$5:$E$79,"Pendiente")</f>
         <v/>
       </c>
       <c r="F6" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"03.??.??",TAREAS!$E$5:$E$77,"Bloqueada")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"03.??.??",TAREAS!$E$5:$E$79,"Bloqueada")</f>
         <v/>
       </c>
       <c r="G6" s="6">
@@ -835,23 +835,23 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"04.??.??")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"04.??.??")</f>
         <v/>
       </c>
       <c r="C7" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"04.??.??",TAREAS!$E$5:$E$77,"Hecha")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"04.??.??",TAREAS!$E$5:$E$79,"Hecha")</f>
         <v/>
       </c>
       <c r="D7" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"04.??.??",TAREAS!$E$5:$E$77,"En curso")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"04.??.??",TAREAS!$E$5:$E$79,"En curso")</f>
         <v/>
       </c>
       <c r="E7" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"04.??.??",TAREAS!$E$5:$E$77,"Pendiente")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"04.??.??",TAREAS!$E$5:$E$79,"Pendiente")</f>
         <v/>
       </c>
       <c r="F7" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"04.??.??",TAREAS!$E$5:$E$77,"Bloqueada")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"04.??.??",TAREAS!$E$5:$E$79,"Bloqueada")</f>
         <v/>
       </c>
       <c r="G7" s="6">
@@ -866,23 +866,23 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"05.??.??")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"05.??.??")</f>
         <v/>
       </c>
       <c r="C8" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"05.??.??",TAREAS!$E$5:$E$77,"Hecha")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"05.??.??",TAREAS!$E$5:$E$79,"Hecha")</f>
         <v/>
       </c>
       <c r="D8" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"05.??.??",TAREAS!$E$5:$E$77,"En curso")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"05.??.??",TAREAS!$E$5:$E$79,"En curso")</f>
         <v/>
       </c>
       <c r="E8" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"05.??.??",TAREAS!$E$5:$E$77,"Pendiente")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"05.??.??",TAREAS!$E$5:$E$79,"Pendiente")</f>
         <v/>
       </c>
       <c r="F8" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"05.??.??",TAREAS!$E$5:$E$77,"Bloqueada")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"05.??.??",TAREAS!$E$5:$E$79,"Bloqueada")</f>
         <v/>
       </c>
       <c r="G8" s="6">
@@ -897,23 +897,23 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"06.??.??")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"06.??.??")</f>
         <v/>
       </c>
       <c r="C9" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"06.??.??",TAREAS!$E$5:$E$77,"Hecha")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"06.??.??",TAREAS!$E$5:$E$79,"Hecha")</f>
         <v/>
       </c>
       <c r="D9" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"06.??.??",TAREAS!$E$5:$E$77,"En curso")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"06.??.??",TAREAS!$E$5:$E$79,"En curso")</f>
         <v/>
       </c>
       <c r="E9" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"06.??.??",TAREAS!$E$5:$E$77,"Pendiente")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"06.??.??",TAREAS!$E$5:$E$79,"Pendiente")</f>
         <v/>
       </c>
       <c r="F9" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"06.??.??",TAREAS!$E$5:$E$77,"Bloqueada")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"06.??.??",TAREAS!$E$5:$E$79,"Bloqueada")</f>
         <v/>
       </c>
       <c r="G9" s="6">
@@ -928,23 +928,23 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"07.??.??")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"07.??.??")</f>
         <v/>
       </c>
       <c r="C10" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"07.??.??",TAREAS!$E$5:$E$77,"Hecha")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"07.??.??",TAREAS!$E$5:$E$79,"Hecha")</f>
         <v/>
       </c>
       <c r="D10" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"07.??.??",TAREAS!$E$5:$E$77,"En curso")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"07.??.??",TAREAS!$E$5:$E$79,"En curso")</f>
         <v/>
       </c>
       <c r="E10" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"07.??.??",TAREAS!$E$5:$E$77,"Pendiente")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"07.??.??",TAREAS!$E$5:$E$79,"Pendiente")</f>
         <v/>
       </c>
       <c r="F10" s="5">
-        <f>COUNTIFS(TAREAS!$A$5:$A$77,"07.??.??",TAREAS!$E$5:$E$77,"Bloqueada")</f>
+        <f>COUNTIFS(TAREAS!$A$5:$A$79,"07.??.??",TAREAS!$E$5:$E$79,"Bloqueada")</f>
         <v/>
       </c>
       <c r="G10" s="6">
@@ -1428,7 +1428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I48"/>
+  <dimension ref="A1:I50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1527,7 +1527,7 @@
       <c r="B6" s="30" t="n"/>
       <c r="C6" s="31" t="inlineStr">
         <is>
-          <t>04.02.01 — Barrido de fuentes: papers, libros, foros, GitHub, X. Regla: mínimo 2 fuentes independientes verificables por idea; vendedores de cursos/señales no son fuente. Detras de ella esperan 16 de las 36 tareas vivas.</t>
+          <t>04.02.01 — Barrido de fuentes: papers, libros, foros, GitHub, X. Regla: mínimo 2 fuentes independientes verificables por idea; vendedores de cursos/señales no son fuente. Detras de ella esperan 16 de las 38 tareas vivas.</t>
         </is>
       </c>
       <c r="D6" s="30" t="n"/>
@@ -1591,7 +1591,7 @@
     <row r="9">
       <c r="A9" s="32" t="inlineStr">
         <is>
-          <t>SE PUEDE TRABAJAR YA — 15 tareas, en este orden</t>
+          <t>SE PUEDE TRABAJAR YA — 16 tareas, en este orden</t>
         </is>
       </c>
       <c r="B9" s="32" t="n"/>
@@ -1711,10 +1711,10 @@
         </is>
       </c>
       <c r="G12" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
@@ -2114,17 +2114,17 @@
       </c>
       <c r="B23" s="33" t="inlineStr">
         <is>
-          <t>07.01.01</t>
+          <t>03.01.25</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Carpetas y documentos en orden; una fuente de verdad por tema; lo sustituido se borra</t>
+          <t>NUEVA 05/08 (nace del incidente de este mismo día): guardia en .githooks/pre-commit que ejecuta la métrica de L-027 de 00-direccion/LECCIONES.md sobre 00-direccion/WBS.md y rechaza el commit si alguna fila de tarea no da 7 campos al partirla por la barra vertical. Motivo: hoy la métrica existe, está escrita como normativa en este WBS, y no la ejecuta nadie automáticamente; 05-vista-ceo/verificar_excel.py no la cubre. Es el muro que le falta a la única fuente de verdad del proyecto. Regla 24 de CLAUDE.md: nace de un incidente real y medido — el 05/08 cuatro filas quedaron partidas y ningún guardia se enteró. Regla 25 de CLAUDE.md: se verifica por inyección de una fila rota ANTES de documentarse como activo. AVISO PARA QUIEN LA EJECUTE, medido el mismo día: el propio texto de esta fila no puede contener el comando literal, porque la barra vertical que lleva dentro rompe la fila que describe; el guardia tiene que tolerar esa cita cuando aparezca en prosa fuera de una tabla.</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Constructores</t>
+          <t>Constructor de motor</t>
         </is>
       </c>
       <c r="E23" s="34" t="inlineStr">
@@ -2151,12 +2151,12 @@
       </c>
       <c r="B24" s="33" t="inlineStr">
         <is>
-          <t>07.01.02</t>
+          <t>07.01.01</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Mejoras del motor: SOLO tareas aprobadas en revisión semanal (el motor no manda)</t>
+          <t>Carpetas y documentos en orden; una fuente de verdad por tema; lo sustituido se borra</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -2183,58 +2183,56 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="32" t="inlineStr">
-        <is>
-          <t>ESPERANDO A OTRA TAREA — 21 tareas, en orden de codigo WBS</t>
-        </is>
-      </c>
-      <c r="B25" s="32" t="n"/>
-      <c r="C25" s="32" t="n"/>
-      <c r="D25" s="32" t="n"/>
-      <c r="E25" s="32" t="n"/>
-      <c r="F25" s="32" t="n"/>
-      <c r="G25" s="32" t="n"/>
-      <c r="H25" s="32" t="n"/>
-      <c r="I25" s="32" t="n"/>
+      <c r="A25" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="B25" s="33" t="inlineStr">
+        <is>
+          <t>07.01.02</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Mejoras del motor: SOLO tareas aprobadas en revisión semanal (el motor no manda)</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Constructores</t>
+        </is>
+      </c>
+      <c r="E25" s="34" t="inlineStr">
+        <is>
+          <t>MOTOR</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr"/>
+      <c r="H25" s="5" t="inlineStr"/>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>nada: se puede empezar ya</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B26" s="33" t="inlineStr">
-        <is>
-          <t>03.01.05</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>PRUEBA REAL DEL MOTOR: un día entero de trabajo desatendido de verdad antes de dar la fase por buena</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>Orquestador</t>
-        </is>
-      </c>
-      <c r="E26" s="34" t="inlineStr">
-        <is>
-          <t>MOTOR</t>
-        </is>
-      </c>
-      <c r="F26" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G26" s="5" t="inlineStr"/>
-      <c r="H26" s="5" t="inlineStr"/>
-      <c r="I26" s="4" t="inlineStr">
-        <is>
-          <t>03.01.03 (pendiente, Constructores), 03.01.04 (pendiente, Constructores)</t>
-        </is>
-      </c>
+      <c r="A26" s="32" t="inlineStr">
+        <is>
+          <t>ESPERANDO A OTRA TAREA — 22 tareas, en orden de codigo WBS</t>
+        </is>
+      </c>
+      <c r="B26" s="32" t="n"/>
+      <c r="C26" s="32" t="n"/>
+      <c r="D26" s="32" t="n"/>
+      <c r="E26" s="32" t="n"/>
+      <c r="F26" s="32" t="n"/>
+      <c r="G26" s="32" t="n"/>
+      <c r="H26" s="32" t="n"/>
+      <c r="I26" s="32" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -2244,17 +2242,17 @@
       </c>
       <c r="B27" s="33" t="inlineStr">
         <is>
-          <t>03.01.07</t>
+          <t>03.01.05</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Cola de aprobación del CEO: tabla con desplegable Aprobado / Saltar / Corregir y columna de corrección. Lo aprobado se ejecuta solo; lo corregido se rehace Y la corrección se guarda en LECCIONES.md</t>
+          <t>PRUEBA REAL DEL MOTOR: un día entero de trabajo desatendido de verdad antes de dar la fase por buena</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Secretario</t>
+          <t>Orquestador</t>
         </is>
       </c>
       <c r="E27" s="34" t="inlineStr">
@@ -2271,7 +2269,7 @@
       <c r="H27" s="5" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>03.01.06 (pendiente, Secretario)</t>
+          <t>03.01.03 (pendiente, Constructores), 03.01.04 (pendiente, Constructores)</t>
         </is>
       </c>
     </row>
@@ -2283,17 +2281,17 @@
       </c>
       <c r="B28" s="33" t="inlineStr">
         <is>
-          <t>03.01.11</t>
+          <t>03.01.07</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>NUEVA 31/07 (D-10): guardia del cajon reservado por cifrado. Script cajon_reservado.py: la contraseña solo la tiene el CEO, no se guarda, se pide en cada operacion y nada se descifra a disco</t>
+          <t>Cola de aprobación del CEO: tabla con desplegable Aprobado / Saltar / Corregir y columna de corrección. Lo aprobado se ejecuta solo; lo corregido se rehace Y la corrección se guarda en LECCIONES.md</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Constructores</t>
+          <t>Secretario</t>
         </is>
       </c>
       <c r="E28" s="34" t="inlineStr">
@@ -2301,16 +2299,16 @@
           <t>MOTOR</t>
         </is>
       </c>
-      <c r="F28" s="14" t="inlineStr">
-        <is>
-          <t>En curso</t>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr"/>
       <c r="H28" s="5" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>03.01.08 (en curso, Crítico)</t>
+          <t>03.01.06 (pendiente, Secretario)</t>
         </is>
       </c>
     </row>
@@ -2322,34 +2320,34 @@
       </c>
       <c r="B29" s="33" t="inlineStr">
         <is>
-          <t>04.01.02</t>
+          <t>03.01.11</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Recalcular costes con precios reales del broker (sustituye 02.01.02) REQUISITO AÑADIDO 04/08: al recalcular con precios reales se comprueba que la entidad que publica la tarifa es la misma con la que se opera. Si no coinciden, la cifra vieja no se hereda: se vuelve a medir.</t>
+          <t>NUEVA 31/07 (D-10): guardia del cajon reservado por cifrado. Script cajon_reservado.py: la contraseña solo la tiene el CEO, no se guarda, se pide en cada operacion y nada se descifra a disco</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Constructor datos</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>PRODUCTO</t>
-        </is>
-      </c>
-      <c r="F29" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+          <t>Constructores</t>
+        </is>
+      </c>
+      <c r="E29" s="34" t="inlineStr">
+        <is>
+          <t>MOTOR</t>
+        </is>
+      </c>
+      <c r="F29" s="14" t="inlineStr">
+        <is>
+          <t>En curso</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr"/>
       <c r="H29" s="5" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>04.01.01 (en curso, CEO + Orquestador)</t>
+          <t>03.01.08 (en curso, Crítico)</t>
         </is>
       </c>
     </row>
@@ -2361,22 +2359,22 @@
       </c>
       <c r="B30" s="33" t="inlineStr">
         <is>
-          <t>04.01.03</t>
+          <t>03.01.24</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Histórico limpio partido en 3 cajones: construir (train), ajustar (validación) y RESERVADO bajo llave (OOS, se abre una sola vez por variante). Ningún agente toca el reservado</t>
+          <t>NUEVA 05/08 (nace de los huecos medidos por ejecución en 03.01.08): las tres barreras que hoy NO existen. (a) El patrón Bash( 02-datos/reservado) de .claude/settings.json exige un espacio literal y no cubre la ruta pegada a una comilla, así que una línea de python lo esquiva: sustituirlo por un patrón que cubra cualquier verbo y cualquier forma de escribir la ruta, y probarlo con las TRES formas. (b) Nada impide rm -rf dentro de 02-datos/, y los datos no están en git (regla 27 de CLAUDE.md): no se rehacen deshaciendo un commit, se rehacen volviendo a descargarlos. (c) No hay ninguna barrera de gasto, ni en código ni en configuración; D-26 de 00-direccion/DECISIONES.md deja escrito que --max-budget-usd existe. Regla 24 de CLAUDE.md: las tres nacen de una inyección ejecutada con su salida guardada, no de una sospecha, y ninguna causó daño. Regla 25 de CLAUDE.md: cada barrera nueva se verifica por inyección ANTES de documentarse como activa.</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Constructor datos</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="inlineStr">
-        <is>
-          <t>PRODUCTO</t>
+          <t>Constructores</t>
+        </is>
+      </c>
+      <c r="E30" s="34" t="inlineStr">
+        <is>
+          <t>MOTOR</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
@@ -2384,15 +2382,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="G30" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H30" s="5" t="n">
-        <v>13</v>
-      </c>
+      <c r="G30" s="5" t="inlineStr"/>
+      <c r="H30" s="5" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>04.01.01 (en curso, CEO + Orquestador)</t>
+          <t>03.01.08 (en curso, Crítico)</t>
         </is>
       </c>
     </row>
@@ -2404,17 +2398,17 @@
       </c>
       <c r="B31" s="33" t="inlineStr">
         <is>
-          <t>04.02.02</t>
+          <t>04.01.02</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Ficha por hipótesis: por qué existiría la ventaja, reglas de entrada/salida, mercado y vela. Sin lógica de por qué gana, no entra (nada de probar por probar)</t>
+          <t>Recalcular costes con precios reales del broker (sustituye 02.01.02) REQUISITO AÑADIDO 04/08: al recalcular con precios reales se comprueba que la entidad que publica la tarifa es la misma con la que se opera. Si no coinciden, la cifra vieja no se hereda: se vuelve a medir.</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Investigador</t>
+          <t>Constructor datos</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -2427,15 +2421,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="G31" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H31" s="5" t="n">
-        <v>15</v>
-      </c>
+      <c r="G31" s="5" t="inlineStr"/>
+      <c r="H31" s="5" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>04.02.01 (pendiente, Investigador)</t>
+          <t>04.01.01 (en curso, CEO + Orquestador)</t>
         </is>
       </c>
     </row>
@@ -2447,17 +2437,17 @@
       </c>
       <c r="B32" s="33" t="inlineStr">
         <is>
-          <t>04.02.03</t>
+          <t>04.01.03</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Filtro de sentido: el Validador puntúa y se eligen las 3-5 mejores</t>
+          <t>Histórico limpio partido en 3 cajones: construir (train), ajustar (validación) y RESERVADO bajo llave (OOS, se abre una sola vez por variante). Ningún agente toca el reservado</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Validador</t>
+          <t>Constructor datos</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -2474,11 +2464,11 @@
         <v>1</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>04.02.02 (pendiente, Investigador)</t>
+          <t>04.01.01 (en curso, CEO + Orquestador)</t>
         </is>
       </c>
     </row>
@@ -2490,17 +2480,17 @@
       </c>
       <c r="B33" s="33" t="inlineStr">
         <is>
-          <t>04.02.04</t>
+          <t>04.02.02</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Pre-registro de variantes: cada hipótesis deja escritas sus variantes ANTES de probar (máx. 5-7 por hipótesis). Lo no registrado no se prueba</t>
+          <t>Ficha por hipótesis: por qué existiría la ventaja, reglas de entrada/salida, mercado y vela. Sin lógica de por qué gana, no entra (nada de probar por probar)</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Validador</t>
+          <t>Investigador</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -2517,11 +2507,11 @@
         <v>1</v>
       </c>
       <c r="H33" s="5" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>04.02.03 (pendiente, Validador)</t>
+          <t>04.02.01 (pendiente, Investigador)</t>
         </is>
       </c>
     </row>
@@ -2533,17 +2523,17 @@
       </c>
       <c r="B34" s="33" t="inlineStr">
         <is>
-          <t>04.03.01</t>
+          <t>04.02.03</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Backtest con costes reales sobre el cajón de construir</t>
+          <t>Filtro de sentido: el Validador puntúa y se eligen las 3-5 mejores</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Constructores</t>
+          <t>Validador</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -2560,11 +2550,11 @@
         <v>1</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>04.01.03 (pendiente, Constructor datos), 04.02.04 (pendiente, Validador)</t>
+          <t>04.02.02 (pendiente, Investigador)</t>
         </is>
       </c>
     </row>
@@ -2576,17 +2566,17 @@
       </c>
       <c r="B35" s="33" t="inlineStr">
         <is>
-          <t>04.03.02</t>
+          <t>04.02.04</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Ajuste SOLO con el cajón de validación; lo que no aguanta, muere aquí</t>
+          <t>Pre-registro de variantes: cada hipótesis deja escritas sus variantes ANTES de probar (máx. 5-7 por hipótesis). Lo no registrado no se prueba</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Constructores</t>
+          <t>Validador</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -2603,11 +2593,11 @@
         <v>1</v>
       </c>
       <c r="H35" s="5" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>04.03.01 (pendiente, Constructores)</t>
+          <t>04.02.03 (pendiente, Validador)</t>
         </is>
       </c>
     </row>
@@ -2619,17 +2609,17 @@
       </c>
       <c r="B36" s="33" t="inlineStr">
         <is>
-          <t>04.03.03</t>
+          <t>04.03.01</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Prueba de fuego: UNA sola pasada por variante sobre el cajón reservado (OOS). Repetir sería hacerse trampa</t>
+          <t>Backtest con costes reales sobre el cajón de construir</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Validador</t>
+          <t>Constructores</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -2646,11 +2636,11 @@
         <v>1</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>04.03.02 (pendiente, Constructores)</t>
+          <t>04.01.03 (pendiente, Constructor datos), 04.02.04 (pendiente, Validador)</t>
         </is>
       </c>
     </row>
@@ -2662,17 +2652,17 @@
       </c>
       <c r="B37" s="33" t="inlineStr">
         <is>
-          <t>04.03.04</t>
+          <t>04.03.02</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Robustez: Monte Carlo (barajar el orden de operaciones y meter pequeños cambios miles de veces: ¿aguanta o era suerte?) + walk-forward (repetir el ajuste avanzando en el tiempo)</t>
+          <t>Ajuste SOLO con el cajón de validación; lo que no aguanta, muere aquí</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Validador</t>
+          <t>Constructores</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -2689,11 +2679,11 @@
         <v>1</v>
       </c>
       <c r="H37" s="5" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>04.03.03 (pendiente, Validador)</t>
+          <t>04.03.01 (pendiente, Constructores)</t>
         </is>
       </c>
     </row>
@@ -2705,12 +2695,12 @@
       </c>
       <c r="B38" s="33" t="inlineStr">
         <is>
-          <t>04.03.05</t>
+          <t>04.03.03</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Veredicto pasa/no pasa por variante, con los criterios de G2. Quien construyó no vota</t>
+          <t>Prueba de fuego: UNA sola pasada por variante sobre el cajón reservado (OOS). Repetir sería hacerse trampa</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
@@ -2732,11 +2722,11 @@
         <v>1</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>04.03.04 (pendiente, Validador)</t>
+          <t>04.03.02 (pendiente, Constructores)</t>
         </is>
       </c>
     </row>
@@ -2748,17 +2738,17 @@
       </c>
       <c r="B39" s="33" t="inlineStr">
         <is>
-          <t>04.04.01</t>
+          <t>04.03.04</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Informe de la vuelta: qué pasó, qué murió y por qué. Registro de TODAS las pruebas, también fallidas</t>
+          <t>Robustez: Monte Carlo (barajar el orden de operaciones y meter pequeños cambios miles de veces: ¿aguanta o era suerte?) + walk-forward (repetir el ajuste avanzando en el tiempo)</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Secretario</t>
+          <t>Validador</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -2772,14 +2762,14 @@
         </is>
       </c>
       <c r="G39" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H39" s="5" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>04.03.05 (pendiente, Validador)</t>
+          <t>04.03.03 (pendiente, Validador)</t>
         </is>
       </c>
     </row>
@@ -2791,17 +2781,17 @@
       </c>
       <c r="B40" s="33" t="inlineStr">
         <is>
-          <t>04.04.02</t>
+          <t>04.03.05</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Si ninguna pasa: volver a 04.02 con lecciones (vuelta 2, 3…). Tras la 3ª vuelta sin éxito: revisión completa del planteamiento con el CEO</t>
+          <t>Veredicto pasa/no pasa por variante, con los criterios de G2. Quien construyó no vota</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Orquestador</t>
+          <t>Validador</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -2814,11 +2804,15 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="G40" s="5" t="inlineStr"/>
-      <c r="H40" s="5" t="inlineStr"/>
+      <c r="G40" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H40" s="5" t="n">
+        <v>8</v>
+      </c>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>04.04.01 (pendiente, Secretario)</t>
+          <t>04.03.04 (pendiente, Validador)</t>
         </is>
       </c>
     </row>
@@ -2830,17 +2824,17 @@
       </c>
       <c r="B41" s="33" t="inlineStr">
         <is>
-          <t>04.04.03</t>
+          <t>04.04.01</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>PUERTA G2: el CEO decide qué pasa a demo</t>
-        </is>
-      </c>
-      <c r="D41" s="28" t="inlineStr">
-        <is>
-          <t>CEO</t>
+          <t>Informe de la vuelta: qué pasó, qué murió y por qué. Registro de TODAS las pruebas, también fallidas</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Secretario</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -2854,14 +2848,14 @@
         </is>
       </c>
       <c r="G41" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H41" s="5" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>04.04.01 (pendiente, Secretario)</t>
+          <t>04.03.05 (pendiente, Validador)</t>
         </is>
       </c>
     </row>
@@ -2873,17 +2867,17 @@
       </c>
       <c r="B42" s="33" t="inlineStr">
         <is>
-          <t>05.01.01</t>
+          <t>04.04.02</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Bot en demo, solo y con guardias automáticos</t>
+          <t>Si ninguna pasa: volver a 04.02 con lecciones (vuelta 2, 3…). Tras la 3ª vuelta sin éxito: revisión completa del planteamiento con el CEO</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Constructores</t>
+          <t>Orquestador</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -2896,15 +2890,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="G42" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H42" s="5" t="n">
-        <v>4</v>
-      </c>
+      <c r="G42" s="5" t="inlineStr"/>
+      <c r="H42" s="5" t="inlineStr"/>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>04.04.03 (pendiente, CEO)</t>
+          <t>04.04.01 (pendiente, Secretario)</t>
         </is>
       </c>
     </row>
@@ -2916,17 +2906,17 @@
       </c>
       <c r="B43" s="33" t="inlineStr">
         <is>
-          <t>05.01.02</t>
+          <t>04.04.03</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Seguimiento semanal real vs. prometido (8-12 semanas)</t>
-        </is>
-      </c>
-      <c r="D43" s="4" t="inlineStr">
-        <is>
-          <t>Secretario</t>
+          <t>PUERTA G2: el CEO decide qué pasa a demo</t>
+        </is>
+      </c>
+      <c r="D43" s="28" t="inlineStr">
+        <is>
+          <t>CEO</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -2943,11 +2933,11 @@
         <v>1</v>
       </c>
       <c r="H43" s="5" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>05.01.01 (pendiente, Constructores)</t>
+          <t>04.04.01 (pendiente, Secretario)</t>
         </is>
       </c>
     </row>
@@ -2959,17 +2949,17 @@
       </c>
       <c r="B44" s="33" t="inlineStr">
         <is>
-          <t>05.01.03</t>
+          <t>05.01.01</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>PUERTA G3: CEO decide dinero, cuánto y pérdida máxima</t>
-        </is>
-      </c>
-      <c r="D44" s="28" t="inlineStr">
-        <is>
-          <t>CEO</t>
+          <t>Bot en demo, solo y con guardias automáticos</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Constructores</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -2986,11 +2976,11 @@
         <v>1</v>
       </c>
       <c r="H44" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>05.01.02 (pendiente, Secretario)</t>
+          <t>04.04.03 (pendiente, CEO)</t>
         </is>
       </c>
     </row>
@@ -3002,17 +2992,17 @@
       </c>
       <c r="B45" s="33" t="inlineStr">
         <is>
-          <t>06.01.01</t>
+          <t>05.01.02</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Dinero pequeño respetando los límites de 01.01.03</t>
+          <t>Seguimiento semanal real vs. prometido (8-12 semanas)</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Constructores</t>
+          <t>Secretario</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -3029,11 +3019,11 @@
         <v>1</v>
       </c>
       <c r="H45" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>05.01.03 (pendiente, CEO)</t>
+          <t>05.01.01 (pendiente, Constructores)</t>
         </is>
       </c>
     </row>
@@ -3045,56 +3035,142 @@
       </c>
       <c r="B46" s="33" t="inlineStr">
         <is>
+          <t>05.01.03</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>PUERTA G3: CEO decide dinero, cuánto y pérdida máxima</t>
+        </is>
+      </c>
+      <c r="D46" s="28" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>PRODUCTO</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H46" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I46" s="4" t="inlineStr">
+        <is>
+          <t>05.01.02 (pendiente, Secretario)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B47" s="33" t="inlineStr">
+        <is>
+          <t>06.01.01</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>Dinero pequeño respetando los límites de 01.01.03</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>Constructores</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>PRODUCTO</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H47" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I47" s="4" t="inlineStr">
+        <is>
+          <t>05.01.03 (pendiente, CEO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B48" s="33" t="inlineStr">
+        <is>
           <t>06.01.02</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr">
+      <c r="C48" s="4" t="inlineStr">
         <is>
           <t>PUERTA G4 mensual: seguir, ampliar o parar. Si pierde más de lo escrito, se para sin discusión</t>
         </is>
       </c>
-      <c r="D46" s="28" t="inlineStr">
+      <c r="D48" s="28" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="E46" s="5" t="inlineStr">
+      <c r="E48" s="5" t="inlineStr">
         <is>
           <t>PRODUCTO</t>
         </is>
       </c>
-      <c r="F46" s="5" t="inlineStr">
+      <c r="F48" s="5" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="G46" s="5" t="inlineStr"/>
-      <c r="H46" s="5" t="inlineStr"/>
-      <c r="I46" s="4" t="inlineStr">
+      <c r="G48" s="5" t="inlineStr"/>
+      <c r="H48" s="5" t="inlineStr"/>
+      <c r="I48" s="4" t="inlineStr">
         <is>
           <t>06.01.01 (pendiente, Constructores)</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="46" customHeight="1">
-      <c r="A48" s="35" t="inlineStr">
-        <is>
-          <t>Aviso de la regla 8 (CLAUDE.md): si la cola de arriba solo tuviera tareas de MOTOR, hay que parar y avisar al CEO; significa que la cola esta mal llena. Ahora mismo la cola tiene 3 de producto y 12 de motor.</t>
+    <row r="50" ht="46" customHeight="1">
+      <c r="A50" s="35" t="inlineStr">
+        <is>
+          <t>Aviso de la regla 8 (CLAUDE.md): si la cola de arriba solo tuviera tareas de MOTOR, hay que parar y avisar al CEO; significa que la cola esta mal llena. Ahora mismo la cola tiene 3 de producto y 13 de motor.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A26:I26"/>
     <mergeCell ref="C6:H6"/>
-    <mergeCell ref="A25:I25"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="C5:H5"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A9:I9"/>
     <mergeCell ref="C4:H4"/>
-    <mergeCell ref="A48:I48"/>
+    <mergeCell ref="A50:I50"/>
     <mergeCell ref="A6:B6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3107,7 +3183,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G77"/>
+  <dimension ref="A1:G79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4477,266 +4553,274 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="36" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="13" t="inlineStr">
+        <is>
+          <t>03.01.24</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>NUEVA 05/08 (nace de los huecos medidos por ejecución en 03.01.08): las tres barreras que hoy NO existen. (a) El patrón Bash( 02-datos/reservado) de .claude/settings.json exige un espacio literal y no cubre la ruta pegada a una comilla, así que una línea de python lo esquiva: sustituirlo por un patrón que cubra cualquier verbo y cualquier forma de escribir la ruta, y probarlo con las TRES formas. (b) Nada impide rm -rf dentro de 02-datos/, y los datos no están en git (regla 27 de CLAUDE.md): no se rehacen deshaciendo un commit, se rehacen volviendo a descargarlos. (c) No hay ninguna barrera de gasto, ni en código ni en configuración; D-26 de 00-direccion/DECISIONES.md deja escrito que --max-budget-usd existe. Regla 24 de CLAUDE.md: las tres nacen de una inyección ejecutada con su salida guardada, no de una sospecha, y ninguna causó daño. Regla 25 de CLAUDE.md: cada barrera nueva se verifica por inyección ANTES de documentarse como activa.</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Constructores</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>03.01.08</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>DESCONGELADA 12/08/2026 por D-36 de 00-direccion/DECISIONES.md, que da la letra aparte que D-29 exigia para aplicar el parche. Ficha de decisión preparada para el 06/08 FICHA ESCRITA Y ENTREGADA 06/08: 00-direccion/informes/FICHA_D-29.md, dos rondas, ACEPTA CON REPAROS de critico-codigo en la ronda 2, con sus dos reparos resueltos antes de cerrar. Los puntos (a), (b) y (c) de esta tarea son los puntos (a), (b) y (c) de la ficha. CORRECCIÓN DE ALCANCE QUE SALIÓ DE LA REVISIÓN, sobre (c): D-26 avisa de que --max-budget-usd puede ser inerte, y la celda de 03.01.23 lo da por medido —no hay clave de API en esta máquina y un tope en dólares no limita nada—, así que (c) puede resultar imposible […] texto completo en 00-direccion/WBS.md</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="13" t="inlineStr">
+        <is>
+          <t>03.01.25</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>NUEVA 05/08 (nace del incidente de este mismo día): guardia en .githooks/pre-commit que ejecuta la métrica de L-027 de 00-direccion/LECCIONES.md sobre 00-direccion/WBS.md y rechaza el commit si alguna fila de tarea no da 7 campos al partirla por la barra vertical. Motivo: hoy la métrica existe, está escrita como normativa en este WBS, y no la ejecuta nadie automáticamente; 05-vista-ceo/verificar_excel.py no la cubre. Es el muro que le falta a la única fuente de verdad del proyecto. Regla 24 de CLAUDE.md: nace de un incidente real y medido — el 05/08 cuatro filas quedaron partidas y ningún guardia se enteró. Regla 25 de CLAUDE.md: se verifica por inyección de una fila rota ANTES de documentarse como activo. AVISO PARA QUIEN LA EJECUTE, medido el mismo día: el propio texto de esta fila no puede contener el comando literal, porque la barra vertical que lleva dentro rompe la fila que describe; el guardia tiene que tolerar esa cita cuando aparezca en prosa fuera de una tabla.</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>Constructor de motor</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>03.01.01</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>DESCONGELADA 12/08/2026 por D-36 de 00-direccion/DECISIONES.md, que da la letra aparte que D-29 exigia para aplicar el parche. Entra como cuarto punto de la ficha D-29 del 06/08 CUMPLIDO 06/08: entra como punto (d) de 00-direccion/informes/FICHA_D-29.md, con la cifra restituida —el 05/08 se partieron cuatro filas— después de que un primer intento la perdiera al apretar prosa; la cazó critico-codigo (L-023 y L-034 de LECCIONES.md). SIGUE pendiente: no se ejecuta hasta que el CEO responda la letra.** Misma advertencia de cita que en 03.01.24: la ficha D-29 no está firmada en DECISIONES.md.</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr"/>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="36" t="inlineStr">
         <is>
           <t>04</t>
         </is>
       </c>
-      <c r="B44" s="37" t="inlineStr">
+      <c r="B46" s="37" t="inlineStr">
         <is>
           <t>HIPÓTESIS Y VALIDACIÓN (PUERTA G2)</t>
         </is>
       </c>
-      <c r="C44" s="37" t="n"/>
-      <c r="D44" s="37" t="n"/>
-      <c r="E44" s="37" t="n"/>
-      <c r="F44" s="37" t="n"/>
-      <c r="G44" s="37" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="38" t="inlineStr">
+      <c r="C46" s="37" t="n"/>
+      <c r="D46" s="37" t="n"/>
+      <c r="E46" s="37" t="n"/>
+      <c r="F46" s="37" t="n"/>
+      <c r="G46" s="37" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="38" t="inlineStr">
         <is>
           <t>04.01</t>
         </is>
       </c>
-      <c r="B45" s="39" t="inlineStr">
+      <c r="B47" s="39" t="inlineStr">
         <is>
           <t>Broker y cajones de datos</t>
         </is>
       </c>
-      <c r="C45" s="39" t="n"/>
-      <c r="D45" s="39" t="n"/>
-      <c r="E45" s="39" t="n"/>
-      <c r="F45" s="39" t="n"/>
-      <c r="G45" s="39" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="13" t="inlineStr">
-        <is>
-          <t>04.01.01</t>
-        </is>
-      </c>
-      <c r="B46" s="4" t="inlineStr">
-        <is>
-          <t>Comparar 3-4 brokers del mercado elegido; elegir uno y abrir demo (CEO firma)</t>
-        </is>
-      </c>
-      <c r="C46" s="28" t="inlineStr">
-        <is>
-          <t>CEO + Orquestador</t>
-        </is>
-      </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>02.03.03</t>
-        </is>
-      </c>
-      <c r="E46" s="4" t="inlineStr">
-        <is>
-          <t>En curso</t>
-        </is>
-      </c>
-      <c r="F46" s="4" t="inlineStr">
-        <is>
-          <t>** 06/08 — comparacion de brokers: ronda 2 cerrada en falso, con una cita literal falsa cazada → 00-direccion/expedientes/04.01.01.md</t>
-        </is>
-      </c>
-      <c r="G46" s="4" t="inlineStr">
-        <is>
-          <t>FICHA (04/08, dictada por el orquestador): Por qué ahora: 02.03.03 cerró el 03/08 con D-19 y esta tarea quedó desbloqueada; es la única con plazo duro —10/08, sin retorno— y quedan 6 días. Alcance: comparar 3 o 4 brokers que ofrezcan XAUUSD al contado y entregar la tabla para que el CEO firme. PROHIBIDO ELEGIR: la elección es del CEO. Criterios obligatorios, uno por columna: (1) lote mínimo, y si admite fraccionado de 0,1 onzas —es eliminatorio de hecho: el lote entero son unos 1.962 € contra […] texto completo en 00-direccion/expedientes/04.01.01.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="13" t="inlineStr">
-        <is>
-          <t>04.01.02</t>
-        </is>
-      </c>
-      <c r="B47" s="4" t="inlineStr">
-        <is>
-          <t>Recalcular costes con precios reales del broker (sustituye 02.01.02) REQUISITO AÑADIDO 04/08: al recalcular con precios reales se comprueba que la entidad que publica la tarifa es la misma con la que se opera. Si no coinciden, la cifra vieja no se hereda: se vuelve a medir.</t>
-        </is>
-      </c>
-      <c r="C47" s="4" t="inlineStr">
-        <is>
-          <t>Constructor datos</t>
-        </is>
-      </c>
-      <c r="D47" s="4" t="inlineStr">
-        <is>
-          <t>04.01.01</t>
-        </is>
-      </c>
-      <c r="E47" s="4" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr"/>
-      <c r="G47" s="4" t="inlineStr"/>
+      <c r="C47" s="39" t="n"/>
+      <c r="D47" s="39" t="n"/>
+      <c r="E47" s="39" t="n"/>
+      <c r="F47" s="39" t="n"/>
+      <c r="G47" s="39" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>04.01.03</t>
+          <t>04.01.01</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>Histórico limpio partido en 3 cajones: construir (train), ajustar (validación) y RESERVADO bajo llave (OOS, se abre una sola vez por variante). Ningún agente toca el reservado</t>
-        </is>
-      </c>
-      <c r="C48" s="4" t="inlineStr">
-        <is>
-          <t>Constructor datos</t>
+          <t>Comparar 3-4 brokers del mercado elegido; elegir uno y abrir demo (CEO firma)</t>
+        </is>
+      </c>
+      <c r="C48" s="28" t="inlineStr">
+        <is>
+          <t>CEO + Orquestador</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>04.01.01</t>
+          <t>02.03.03</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F48" s="4" t="inlineStr"/>
-      <c r="G48" s="4" t="inlineStr"/>
+          <t>En curso</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>** 06/08 — comparacion de brokers: ronda 2 cerrada en falso, con una cita literal falsa cazada → 00-direccion/expedientes/04.01.01.md</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>FICHA (04/08, dictada por el orquestador): Por qué ahora: 02.03.03 cerró el 03/08 con D-19 y esta tarea quedó desbloqueada; es la única con plazo duro —10/08, sin retorno— y quedan 6 días. Alcance: comparar 3 o 4 brokers que ofrezcan XAUUSD al contado y entregar la tabla para que el CEO firme. PROHIBIDO ELEGIR: la elección es del CEO. Criterios obligatorios, uno por columna: (1) lote mínimo, y si admite fraccionado de 0,1 onzas —es eliminatorio de hecho: el lote entero son unos 1.962 € contra […] texto completo en 00-direccion/expedientes/04.01.01.md</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="13" t="inlineStr">
         <is>
-          <t>04.01.04</t>
+          <t>04.01.02</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>NUEVA 09/08 (subtarea dentro del alcance de 04.01.01, creada por el orquestador, regla 2 de CLAUDE.md): re-derivar POR CÁLCULO el tamaño mínimo operable de XAUUSD en 4h y el requisito real de lote que 04.01.01 debe exigir al bróker</t>
+          <t>Recalcular costes con precios reales del broker (sustituye 02.01.02) REQUISITO AÑADIDO 04/08: al recalcular con precios reales se comprueba que la entidad que publica la tarifa es la misma con la que se opera. Si no coinciden, la cifra vieja no se hereda: se vuelve a medir.</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Constructor de datos</t>
+          <t>Constructor datos</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>02.02.01, 02.03.03</t>
+          <t>04.01.01</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>En curso</t>
-        </is>
-      </c>
-      <c r="F49" s="4" t="inlineStr">
-        <is>
-          <t>** 09/08 — re-derivacion de la comparacion de brokers; ficha escrita tarde y anotada como incumplimiento → 00-direccion/expedientes/04.01.04.md</t>
-        </is>
-      </c>
-      <c r="G49" s="4" t="inlineStr">
-        <is>
-          <t>en_curso — FICHA ESCRITA TARDE Y POR ESO ANOTADA (regla 5 de CLAUDE.md incumplida): el orquestador dictó esta subtarea en el reparto del 09/08 con código, motivo y criterio de hecho, pero ordenó ejecutarla sin mandar que se escribiera antes en este WBS; el trabajo se hizo el mismo día y la fila se añade después. Lo detectó validador al revisar la entrega, con grep -rn "04.01.04" 00-direccion/ devolviendo cero. Es el defecto de L-013 de LECCIONES.md, ya anotado en las celdas de 01.02.03 y […] texto completo en 00-direccion/expedientes/04.01.04.md</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr"/>
+      <c r="G49" s="4" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="38" t="inlineStr">
-        <is>
-          <t>04.02</t>
-        </is>
-      </c>
-      <c r="B50" s="39" t="inlineStr">
-        <is>
-          <t>Investigación de hipótesis</t>
-        </is>
-      </c>
-      <c r="C50" s="39" t="n"/>
-      <c r="D50" s="39" t="n"/>
-      <c r="E50" s="39" t="n"/>
-      <c r="F50" s="39" t="n"/>
-      <c r="G50" s="39" t="n"/>
+      <c r="A50" s="13" t="inlineStr">
+        <is>
+          <t>04.01.03</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Histórico limpio partido en 3 cajones: construir (train), ajustar (validación) y RESERVADO bajo llave (OOS, se abre una sola vez por variante). Ningún agente toca el reservado</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>Constructor datos</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>04.01.01</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr"/>
+      <c r="G50" s="4" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="13" t="inlineStr">
         <is>
-          <t>04.02.01</t>
+          <t>04.01.04</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>Barrido de fuentes: papers, libros, foros, GitHub, X. Regla: mínimo 2 fuentes independientes verificables por idea; vendedores de cursos/señales no son fuente</t>
+          <t>NUEVA 09/08 (subtarea dentro del alcance de 04.01.01, creada por el orquestador, regla 2 de CLAUDE.md): re-derivar POR CÁLCULO el tamaño mínimo operable de XAUUSD en 4h y el requisito real de lote que 04.01.01 debe exigir al bróker</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Investigador</t>
+          <t>Constructor de datos</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>03.01.02</t>
+          <t>02.02.01, 02.03.03</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F51" s="4" t="inlineStr"/>
-      <c r="G51" s="4" t="inlineStr"/>
+          <t>En curso</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>** 09/08 — re-derivacion de la comparacion de brokers; ficha escrita tarde y anotada como incumplimiento → 00-direccion/expedientes/04.01.04.md</t>
+        </is>
+      </c>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>en_curso — FICHA ESCRITA TARDE Y POR ESO ANOTADA (regla 5 de CLAUDE.md incumplida): el orquestador dictó esta subtarea en el reparto del 09/08 con código, motivo y criterio de hecho, pero ordenó ejecutarla sin mandar que se escribiera antes en este WBS; el trabajo se hizo el mismo día y la fila se añade después. Lo detectó validador al revisar la entrega, con grep -rn "04.01.04" 00-direccion/ devolviendo cero. Es el defecto de L-013 de LECCIONES.md, ya anotado en las celdas de 01.02.03 y […] texto completo en 00-direccion/expedientes/04.01.04.md</t>
+        </is>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" s="13" t="inlineStr">
-        <is>
-          <t>04.02.02</t>
-        </is>
-      </c>
-      <c r="B52" s="4" t="inlineStr">
-        <is>
-          <t>Ficha por hipótesis: por qué existiría la ventaja, reglas de entrada/salida, mercado y vela. Sin lógica de por qué gana, no entra (nada de probar por probar)</t>
-        </is>
-      </c>
-      <c r="C52" s="4" t="inlineStr">
-        <is>
-          <t>Investigador</t>
-        </is>
-      </c>
-      <c r="D52" s="4" t="inlineStr">
-        <is>
-          <t>04.02.01</t>
-        </is>
-      </c>
-      <c r="E52" s="4" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F52" s="4" t="inlineStr"/>
-      <c r="G52" s="4" t="inlineStr"/>
+      <c r="A52" s="38" t="inlineStr">
+        <is>
+          <t>04.02</t>
+        </is>
+      </c>
+      <c r="B52" s="39" t="inlineStr">
+        <is>
+          <t>Investigación de hipótesis</t>
+        </is>
+      </c>
+      <c r="C52" s="39" t="n"/>
+      <c r="D52" s="39" t="n"/>
+      <c r="E52" s="39" t="n"/>
+      <c r="F52" s="39" t="n"/>
+      <c r="G52" s="39" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="13" t="inlineStr">
         <is>
-          <t>04.02.03</t>
+          <t>04.02.01</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>Filtro de sentido: el Validador puntúa y se eligen las 3-5 mejores</t>
+          <t>Barrido de fuentes: papers, libros, foros, GitHub, X. Regla: mínimo 2 fuentes independientes verificables por idea; vendedores de cursos/señales no son fuente</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Validador</t>
+          <t>Investigador</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>04.02.02</t>
+          <t>03.01.02</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
@@ -4750,22 +4834,22 @@
     <row r="54">
       <c r="A54" s="13" t="inlineStr">
         <is>
-          <t>04.02.04</t>
+          <t>04.02.02</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>Pre-registro de variantes: cada hipótesis deja escritas sus variantes ANTES de probar (máx. 5-7 por hipótesis). Lo no registrado no se prueba</t>
+          <t>Ficha por hipótesis: por qué existiría la ventaja, reglas de entrada/salida, mercado y vela. Sin lógica de por qué gana, no entra (nada de probar por probar)</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Validador</t>
+          <t>Investigador</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>04.02.03</t>
+          <t>04.02.01</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
@@ -4777,41 +4861,53 @@
       <c r="G54" s="4" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" s="38" t="inlineStr">
-        <is>
-          <t>04.03</t>
-        </is>
-      </c>
-      <c r="B55" s="39" t="inlineStr">
-        <is>
-          <t>Laboratorio de pruebas (por hipótesis y variante)</t>
-        </is>
-      </c>
-      <c r="C55" s="39" t="n"/>
-      <c r="D55" s="39" t="n"/>
-      <c r="E55" s="39" t="n"/>
-      <c r="F55" s="39" t="n"/>
-      <c r="G55" s="39" t="n"/>
+      <c r="A55" s="13" t="inlineStr">
+        <is>
+          <t>04.02.03</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>Filtro de sentido: el Validador puntúa y se eligen las 3-5 mejores</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>Validador</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>04.02.02</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr"/>
+      <c r="G55" s="4" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="13" t="inlineStr">
         <is>
-          <t>04.03.01</t>
+          <t>04.02.04</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>Backtest con costes reales sobre el cajón de construir</t>
+          <t>Pre-registro de variantes: cada hipótesis deja escritas sus variantes ANTES de probar (máx. 5-7 por hipótesis). Lo no registrado no se prueba</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Constructores</t>
+          <t>Validador</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>04.01.03, 04.02.04, 04.03.07</t>
+          <t>04.02.03</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
@@ -4823,53 +4919,41 @@
       <c r="G56" s="4" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="13" t="inlineStr">
-        <is>
-          <t>04.03.02</t>
-        </is>
-      </c>
-      <c r="B57" s="4" t="inlineStr">
-        <is>
-          <t>Ajuste SOLO con el cajón de validación; lo que no aguanta, muere aquí</t>
-        </is>
-      </c>
-      <c r="C57" s="4" t="inlineStr">
-        <is>
-          <t>Constructores</t>
-        </is>
-      </c>
-      <c r="D57" s="4" t="inlineStr">
-        <is>
-          <t>04.03.01</t>
-        </is>
-      </c>
-      <c r="E57" s="4" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F57" s="4" t="inlineStr"/>
-      <c r="G57" s="4" t="inlineStr"/>
+      <c r="A57" s="38" t="inlineStr">
+        <is>
+          <t>04.03</t>
+        </is>
+      </c>
+      <c r="B57" s="39" t="inlineStr">
+        <is>
+          <t>Laboratorio de pruebas (por hipótesis y variante)</t>
+        </is>
+      </c>
+      <c r="C57" s="39" t="n"/>
+      <c r="D57" s="39" t="n"/>
+      <c r="E57" s="39" t="n"/>
+      <c r="F57" s="39" t="n"/>
+      <c r="G57" s="39" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="13" t="inlineStr">
         <is>
-          <t>04.03.03</t>
+          <t>04.03.01</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>Prueba de fuego: UNA sola pasada por variante sobre el cajón reservado (OOS). Repetir sería hacerse trampa</t>
+          <t>Backtest con costes reales sobre el cajón de construir</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>Validador</t>
+          <t>Constructores</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>04.03.02</t>
+          <t>04.01.03, 04.02.04, 04.03.07</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
@@ -4883,22 +4967,22 @@
     <row r="59">
       <c r="A59" s="13" t="inlineStr">
         <is>
-          <t>04.03.04</t>
+          <t>04.03.02</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>Robustez: Monte Carlo (barajar el orden de operaciones y meter pequeños cambios miles de veces: ¿aguanta o era suerte?) + walk-forward (repetir el ajuste avanzando en el tiempo)</t>
+          <t>Ajuste SOLO con el cajón de validación; lo que no aguanta, muere aquí</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>Validador</t>
+          <t>Constructores</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>04.03.03</t>
+          <t>04.03.01</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
@@ -4912,12 +4996,12 @@
     <row r="60">
       <c r="A60" s="13" t="inlineStr">
         <is>
-          <t>04.03.05</t>
+          <t>04.03.03</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>Veredicto pasa/no pasa por variante, con los criterios de G2. Quien construyó no vota</t>
+          <t>Prueba de fuego: UNA sola pasada por variante sobre el cajón reservado (OOS). Repetir sería hacerse trampa</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
@@ -4927,7 +5011,7 @@
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>04.03.04</t>
+          <t>04.03.02</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
@@ -4941,171 +5025,171 @@
     <row r="61">
       <c r="A61" s="13" t="inlineStr">
         <is>
-          <t>04.03.06</t>
+          <t>04.03.04</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>NUEVA 03/08 (decisión del CEO, opción B): especificación del motor de backtest propio, escrita para una construcción desde cero y no para un trasplante</t>
+          <t>Robustez: Monte Carlo (barajar el orden de operaciones y meter pequeños cambios miles de veces: ¿aguanta o era suerte?) + walk-forward (repetir el ajuste avanzando en el tiempo)</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Arquitecto</t>
+          <t>Validador</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>02.03.03</t>
+          <t>04.03.03</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>Hecha</t>
-        </is>
-      </c>
-      <c r="F61" s="4" t="inlineStr">
-        <is>
-          <t>** 04/08 — especificacion del motor de backtest: 16 requisitos con prueba ejecutable y 8 casos a mano → 00-direccion/expedientes/04.03.06.md</t>
-        </is>
-      </c>
-      <c r="G61" s="4" t="inlineStr">
-        <is>
-          <t>FICHA (03/08, dictada por el orquestador): Por qué se rehace y no se rescata: el criterio de aceptación anterior vivía en la sección «Trasplante desde gb2 — criterios de aceptación», que la cirugía de D-21 borró y hoy solo existe en el historial de git. Nació describiendo qué se traía y qué se descartaba de otro proyecto, y se escribió el 30/07, antes de D-19 y antes de las mediciones de la Fase 02, así que no dice nada del oro, ni de la vela de 4h, ni del lote mínimo. Insumos obligatorios: los […] texto completo en 00-direccion/expedientes/04.03.06.md</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr"/>
+      <c r="G61" s="4" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="13" t="inlineStr">
         <is>
-          <t>04.03.07</t>
+          <t>04.03.05</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>NUEVA 03/08 (decisión del CEO, opción B): construir el motor de backtest desde cero contra la especificación de 04.03.06, tras retirar el anterior</t>
+          <t>Veredicto pasa/no pasa por variante, con los criterios de G2. Quien construyó no vota</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>Constructor de motor</t>
+          <t>Validador</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>04.03.06, 07.01.03</t>
+          <t>04.03.04</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="inlineStr"/>
+      <c r="G62" s="4" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="13" t="inlineStr">
+        <is>
+          <t>04.03.06</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>NUEVA 03/08 (decisión del CEO, opción B): especificación del motor de backtest propio, escrita para una construcción desde cero y no para un trasplante</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>Arquitecto</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>02.03.03</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
           <t>Hecha</t>
         </is>
       </c>
-      <c r="F62" s="4" t="inlineStr">
-        <is>
-          <t>** 04/08 — motor de backtest construido desde cero; procedencia independiente de las dos fuentes → 00-direccion/expedientes/04.03.07.md</t>
-        </is>
-      </c>
-      <c r="G62" s="4" t="inlineStr">
-        <is>
-          <t>FICHA (03/08, dictada por el orquestador): PASO 0, que se ejecuta antes que nada: retirar del árbol de trabajo el motor anterior con git revert, sin reescribir historia, para que quien construya no lo tenga delante. El código sigue existiendo en el commit 0c35959 para siempre, y con él sus 44 funciones de prueba —13 en test_costs.py, 20 en test_execution.py y 11 en test_sizing.py, contadas sobre el commit— que la regla 20 de CLAUDE.md obliga a conservar aunque no se usen. Verificado antes de […] texto completo en 00-direccion/expedientes/04.03.07.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="38" t="inlineStr">
-        <is>
-          <t>04.04</t>
-        </is>
-      </c>
-      <c r="B63" s="39" t="inlineStr">
-        <is>
-          <t>Decisión y bucle</t>
-        </is>
-      </c>
-      <c r="C63" s="39" t="n"/>
-      <c r="D63" s="39" t="n"/>
-      <c r="E63" s="39" t="n"/>
-      <c r="F63" s="39" t="n"/>
-      <c r="G63" s="39" t="n"/>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>** 04/08 — especificacion del motor de backtest: 16 requisitos con prueba ejecutable y 8 casos a mano → 00-direccion/expedientes/04.03.06.md</t>
+        </is>
+      </c>
+      <c r="G63" s="4" t="inlineStr">
+        <is>
+          <t>FICHA (03/08, dictada por el orquestador): Por qué se rehace y no se rescata: el criterio de aceptación anterior vivía en la sección «Trasplante desde gb2 — criterios de aceptación», que la cirugía de D-21 borró y hoy solo existe en el historial de git. Nació describiendo qué se traía y qué se descartaba de otro proyecto, y se escribió el 30/07, antes de D-19 y antes de las mediciones de la Fase 02, así que no dice nada del oro, ni de la vela de 4h, ni del lote mínimo. Insumos obligatorios: los […] texto completo en 00-direccion/expedientes/04.03.06.md</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="13" t="inlineStr">
         <is>
-          <t>04.04.01</t>
+          <t>04.03.07</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>Informe de la vuelta: qué pasó, qué murió y por qué. Registro de TODAS las pruebas, también fallidas</t>
+          <t>NUEVA 03/08 (decisión del CEO, opción B): construir el motor de backtest desde cero contra la especificación de 04.03.06, tras retirar el anterior</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>Secretario</t>
+          <t>Constructor de motor</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>04.03.05</t>
+          <t>04.03.06, 07.01.03</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F64" s="4" t="inlineStr"/>
-      <c r="G64" s="4" t="inlineStr"/>
+          <t>Hecha</t>
+        </is>
+      </c>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t>** 04/08 — motor de backtest construido desde cero; procedencia independiente de las dos fuentes → 00-direccion/expedientes/04.03.07.md</t>
+        </is>
+      </c>
+      <c r="G64" s="4" t="inlineStr">
+        <is>
+          <t>FICHA (03/08, dictada por el orquestador): PASO 0, que se ejecuta antes que nada: retirar del árbol de trabajo el motor anterior con git revert, sin reescribir historia, para que quien construya no lo tenga delante. El código sigue existiendo en el commit 0c35959 para siempre, y con él sus 44 funciones de prueba —13 en test_costs.py, 20 en test_execution.py y 11 en test_sizing.py, contadas sobre el commit— que la regla 20 de CLAUDE.md obliga a conservar aunque no se usen. Verificado antes de […] texto completo en 00-direccion/expedientes/04.03.07.md</t>
+        </is>
+      </c>
     </row>
     <row r="65">
-      <c r="A65" s="13" t="inlineStr">
-        <is>
-          <t>04.04.02</t>
-        </is>
-      </c>
-      <c r="B65" s="4" t="inlineStr">
-        <is>
-          <t>Si ninguna pasa: volver a 04.02 con lecciones (vuelta 2, 3…). Tras la 3ª vuelta sin éxito: revisión completa del planteamiento con el CEO</t>
-        </is>
-      </c>
-      <c r="C65" s="4" t="inlineStr">
-        <is>
-          <t>Orquestador</t>
-        </is>
-      </c>
-      <c r="D65" s="4" t="inlineStr">
-        <is>
-          <t>04.04.01</t>
-        </is>
-      </c>
-      <c r="E65" s="4" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F65" s="4" t="inlineStr"/>
-      <c r="G65" s="4" t="inlineStr"/>
+      <c r="A65" s="38" t="inlineStr">
+        <is>
+          <t>04.04</t>
+        </is>
+      </c>
+      <c r="B65" s="39" t="inlineStr">
+        <is>
+          <t>Decisión y bucle</t>
+        </is>
+      </c>
+      <c r="C65" s="39" t="n"/>
+      <c r="D65" s="39" t="n"/>
+      <c r="E65" s="39" t="n"/>
+      <c r="F65" s="39" t="n"/>
+      <c r="G65" s="39" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="13" t="inlineStr">
         <is>
-          <t>04.04.03</t>
+          <t>04.04.01</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>PUERTA G2: el CEO decide qué pasa a demo</t>
-        </is>
-      </c>
-      <c r="C66" s="28" t="inlineStr">
-        <is>
-          <t>CEO</t>
+          <t>Informe de la vuelta: qué pasó, qué murió y por qué. Registro de TODAS las pruebas, también fallidas</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>Secretario</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>04.04.01</t>
+          <t>04.03.05</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
@@ -5116,42 +5200,54 @@
       <c r="F66" s="4" t="inlineStr"/>
       <c r="G66" s="4" t="inlineStr"/>
     </row>
-    <row r="67" ht="20" customHeight="1">
-      <c r="A67" s="36" t="inlineStr">
-        <is>
-          <t>05</t>
-        </is>
-      </c>
-      <c r="B67" s="37" t="inlineStr">
-        <is>
-          <t>DEMO (PUERTA G3) — SE DETALLA AL CERRAR G2</t>
-        </is>
-      </c>
-      <c r="C67" s="37" t="n"/>
-      <c r="D67" s="37" t="n"/>
-      <c r="E67" s="37" t="n"/>
-      <c r="F67" s="37" t="n"/>
-      <c r="G67" s="37" t="n"/>
+    <row r="67">
+      <c r="A67" s="13" t="inlineStr">
+        <is>
+          <t>04.04.02</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>Si ninguna pasa: volver a 04.02 con lecciones (vuelta 2, 3…). Tras la 3ª vuelta sin éxito: revisión completa del planteamiento con el CEO</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>Orquestador</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>04.04.01</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr"/>
+      <c r="G67" s="4" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="13" t="inlineStr">
         <is>
-          <t>05.01.01</t>
+          <t>04.04.03</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>Bot en demo, solo y con guardias automáticos</t>
-        </is>
-      </c>
-      <c r="C68" s="4" t="inlineStr">
-        <is>
-          <t>Constructores</t>
+          <t>PUERTA G2: el CEO decide qué pasa a demo</t>
+        </is>
+      </c>
+      <c r="C68" s="28" t="inlineStr">
+        <is>
+          <t>CEO</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>04.04.03</t>
+          <t>04.04.01</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
@@ -5159,186 +5255,186 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F68" s="4" t="inlineStr">
-        <is>
-          <t>REQUISITO AÑADIDO POR D-14 (01/08): el guardia de parada dura (-30% del capital inicial) lo aplica el BOT de forma CONTINUA, no una revision periodica; comprobado solo una vez al mes, un -30% puede ser un -45% cuando alguien mire. Se verifica por inyeccion antes de declararlo activo (regla 25 de CLAUDE.md).</t>
-        </is>
-      </c>
+      <c r="F68" s="4" t="inlineStr"/>
       <c r="G68" s="4" t="inlineStr"/>
     </row>
-    <row r="69">
-      <c r="A69" s="13" t="inlineStr">
-        <is>
-          <t>05.01.02</t>
-        </is>
-      </c>
-      <c r="B69" s="4" t="inlineStr">
-        <is>
-          <t>Seguimiento semanal real vs. prometido (8-12 semanas)</t>
-        </is>
-      </c>
-      <c r="C69" s="4" t="inlineStr">
-        <is>
-          <t>Secretario</t>
-        </is>
-      </c>
-      <c r="D69" s="4" t="inlineStr">
-        <is>
-          <t>05.01.01</t>
-        </is>
-      </c>
-      <c r="E69" s="4" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F69" s="4" t="inlineStr"/>
-      <c r="G69" s="4" t="inlineStr"/>
+    <row r="69" ht="20" customHeight="1">
+      <c r="A69" s="36" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="B69" s="37" t="inlineStr">
+        <is>
+          <t>DEMO (PUERTA G3) — SE DETALLA AL CERRAR G2</t>
+        </is>
+      </c>
+      <c r="C69" s="37" t="n"/>
+      <c r="D69" s="37" t="n"/>
+      <c r="E69" s="37" t="n"/>
+      <c r="F69" s="37" t="n"/>
+      <c r="G69" s="37" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="13" t="inlineStr">
         <is>
-          <t>05.01.03</t>
+          <t>05.01.01</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>PUERTA G3: CEO decide dinero, cuánto y pérdida máxima</t>
-        </is>
-      </c>
-      <c r="C70" s="28" t="inlineStr">
-        <is>
-          <t>CEO</t>
+          <t>Bot en demo, solo y con guardias automáticos</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>Constructores</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
+          <t>04.04.03</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>REQUISITO AÑADIDO POR D-14 (01/08): el guardia de parada dura (-30% del capital inicial) lo aplica el BOT de forma CONTINUA, no una revision periodica; comprobado solo una vez al mes, un -30% puede ser un -45% cuando alguien mire. Se verifica por inyeccion antes de declararlo activo (regla 25 de CLAUDE.md).</t>
+        </is>
+      </c>
+      <c r="G70" s="4" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="13" t="inlineStr">
+        <is>
           <t>05.01.02</t>
         </is>
       </c>
-      <c r="E70" s="4" t="inlineStr">
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>Seguimiento semanal real vs. prometido (8-12 semanas)</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>Secretario</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t>05.01.01</t>
+        </is>
+      </c>
+      <c r="E71" s="4" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F70" s="4" t="inlineStr"/>
-      <c r="G70" s="4" t="inlineStr"/>
-    </row>
-    <row r="71" ht="20" customHeight="1">
-      <c r="A71" s="36" t="inlineStr">
-        <is>
-          <t>06</t>
-        </is>
-      </c>
-      <c r="B71" s="37" t="inlineStr">
-        <is>
-          <t>REAL (PUERTA G4) — SE DETALLA AL CERRAR G3</t>
-        </is>
-      </c>
-      <c r="C71" s="37" t="n"/>
-      <c r="D71" s="37" t="n"/>
-      <c r="E71" s="37" t="n"/>
-      <c r="F71" s="37" t="n"/>
-      <c r="G71" s="37" t="n"/>
+      <c r="F71" s="4" t="inlineStr"/>
+      <c r="G71" s="4" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="13" t="inlineStr">
         <is>
+          <t>05.01.03</t>
+        </is>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>PUERTA G3: CEO decide dinero, cuánto y pérdida máxima</t>
+        </is>
+      </c>
+      <c r="C72" s="28" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>05.01.02</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F72" s="4" t="inlineStr"/>
+      <c r="G72" s="4" t="inlineStr"/>
+    </row>
+    <row r="73" ht="20" customHeight="1">
+      <c r="A73" s="36" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="B73" s="37" t="inlineStr">
+        <is>
+          <t>REAL (PUERTA G4) — SE DETALLA AL CERRAR G3</t>
+        </is>
+      </c>
+      <c r="C73" s="37" t="n"/>
+      <c r="D73" s="37" t="n"/>
+      <c r="E73" s="37" t="n"/>
+      <c r="F73" s="37" t="n"/>
+      <c r="G73" s="37" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="13" t="inlineStr">
+        <is>
           <t>06.01.01</t>
         </is>
       </c>
-      <c r="B72" s="4" t="inlineStr">
+      <c r="B74" s="4" t="inlineStr">
         <is>
           <t>Dinero pequeño respetando los límites de 01.01.03</t>
         </is>
       </c>
-      <c r="C72" s="4" t="inlineStr">
+      <c r="C74" s="4" t="inlineStr">
         <is>
           <t>Constructores</t>
         </is>
       </c>
-      <c r="D72" s="4" t="inlineStr">
+      <c r="D74" s="4" t="inlineStr">
         <is>
           <t>05.01.03</t>
         </is>
       </c>
-      <c r="E72" s="4" t="inlineStr">
+      <c r="E74" s="4" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F72" s="4" t="inlineStr">
+      <c r="F74" s="4" t="inlineStr">
         <is>
           <t>limites ya escritos y firmados (D-14, 01/08): capital 1.000-2.000 €, AVISO a -25% del capital inicial que no para nada, PARADA DURA AUTOMATICA a -30% aplicada por el bot de forma continua y sin exencion activable desde dentro (regla 26 de CLAUDE.md).</t>
         </is>
       </c>
-      <c r="G72" s="4" t="inlineStr"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="13" t="inlineStr">
-        <is>
-          <t>06.01.02</t>
-        </is>
-      </c>
-      <c r="B73" s="4" t="inlineStr">
-        <is>
-          <t>PUERTA G4 mensual: seguir, ampliar o parar. Si pierde más de lo escrito, se para sin discusión</t>
-        </is>
-      </c>
-      <c r="C73" s="28" t="inlineStr">
-        <is>
-          <t>CEO</t>
-        </is>
-      </c>
-      <c r="D73" s="4" t="inlineStr">
-        <is>
-          <t>06.01.01</t>
-        </is>
-      </c>
-      <c r="E73" s="4" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F73" s="4" t="inlineStr"/>
-      <c r="G73" s="4" t="inlineStr"/>
-    </row>
-    <row r="74" ht="20" customHeight="1">
-      <c r="A74" s="36" t="inlineStr">
-        <is>
-          <t>07</t>
-        </is>
-      </c>
-      <c r="B74" s="37" t="inlineStr">
-        <is>
-          <t>MOTOR Y ORDEN (PARALELA; MÁX. 20% DEL ESFUERZO SEMANAL)</t>
-        </is>
-      </c>
-      <c r="C74" s="37" t="n"/>
-      <c r="D74" s="37" t="n"/>
-      <c r="E74" s="37" t="n"/>
-      <c r="F74" s="37" t="n"/>
-      <c r="G74" s="37" t="n"/>
+      <c r="G74" s="4" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="13" t="inlineStr">
         <is>
-          <t>07.01.01</t>
+          <t>06.01.02</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>Carpetas y documentos en orden; una fuente de verdad por tema; lo sustituido se borra</t>
-        </is>
-      </c>
-      <c r="C75" s="4" t="inlineStr">
-        <is>
-          <t>Constructores</t>
+          <t>PUERTA G4 mensual: seguir, ampliar o parar. Si pierde más de lo escrito, se para sin discusión</t>
+        </is>
+      </c>
+      <c r="C75" s="28" t="inlineStr">
+        <is>
+          <t>CEO</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>03.01.01</t>
+          <t>06.01.01</t>
         </is>
       </c>
       <c r="E75" s="4" t="inlineStr">
@@ -5346,90 +5442,136 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F75" s="4" t="inlineStr">
-        <is>
-          <t>** 02/08 — orden de carpetas y documentos: la cifra 246/105 retirada por no reproducirse. Sin cerrar → 00-direccion/expedientes/07.01.01.md</t>
-        </is>
-      </c>
-      <c r="G75" s="4" t="inlineStr">
-        <is>
-          <t>FICHA (02/08): ALCANCE — cuatro arreglos de documento, NINGUNO toca código: (a) Las celdas ESTADO de 01.02.04 y 03.01.12 declaran en negrita un estado del vocabulario pendiente / en_curso / hecha / bloqueada, como exige la sección «Estados y cadencia de este WBS». Valores ya decididos por el orquestador, no se deducen: 01.02.04 pasa a en_curso (entregado INFORME_MCP_2.md, RECHAZADO por critico-codigo, sin reparar); 03.01.12 pasa a pendiente (nadie la ha trabajado). En 01.02.04 la marca actual […] texto completo en 00-direccion/expedientes/07.01.01.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="13" t="inlineStr">
-        <is>
-          <t>07.01.03</t>
-        </is>
-      </c>
-      <c r="B76" s="4" t="inlineStr">
-        <is>
-          <t>NUEVA 03/08 (incidente de proceso): auditar todo lo escrito el 03/08/2026 entre las 21:44 y las 21:58 sin flujo de cuatro capas, y el residuo sin commitear del tramo anterior</t>
-        </is>
-      </c>
-      <c r="C76" s="4" t="inlineStr">
-        <is>
-          <t>Orquestador</t>
-        </is>
-      </c>
-      <c r="D76" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E76" s="4" t="inlineStr">
-        <is>
-          <t>En curso</t>
-        </is>
-      </c>
-      <c r="F76" s="4" t="inlineStr">
-        <is>
-          <t>** 09/08 — auditoria de lo escrito sin flujo el 03/08; los lotes de aptitud cancelados por el CEO → 00-direccion/expedientes/07.01.03.md</t>
-        </is>
-      </c>
-      <c r="G76" s="4" t="inlineStr">
-        <is>
-          <t>FICHA (03/08, dictada por el orquestador): Qué pasó, medido y no supuesto: tras un /compact a las 21:29, la sesión recibió una orden del CEO a las 21:44 y trabajó sola hasta las 21:58 sin invocar a un solo subagente. Escribió D-19, D-20 y D-21 en un registro de solo-añadir, L-024 a L-027, cirugía estructural sobre el WBS, y dos scripts del Excel del CEO. Nadie lo revisó (regla 16 de CLAUDE.md y C2 rotas). Alcance: tres lotes con veredicto propio — (d) procedencia del motor de backtest, (b y c) […] texto completo en 00-direccion/expedientes/07.01.03.md</t>
-        </is>
-      </c>
+      <c r="F75" s="4" t="inlineStr"/>
+      <c r="G75" s="4" t="inlineStr"/>
+    </row>
+    <row r="76" ht="20" customHeight="1">
+      <c r="A76" s="36" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="B76" s="37" t="inlineStr">
+        <is>
+          <t>MOTOR Y ORDEN (PARALELA; MÁX. 20% DEL ESFUERZO SEMANAL)</t>
+        </is>
+      </c>
+      <c r="C76" s="37" t="n"/>
+      <c r="D76" s="37" t="n"/>
+      <c r="E76" s="37" t="n"/>
+      <c r="F76" s="37" t="n"/>
+      <c r="G76" s="37" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="13" t="inlineStr">
         <is>
+          <t>07.01.01</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>Carpetas y documentos en orden; una fuente de verdad por tema; lo sustituido se borra</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>Constructores</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>03.01.01</t>
+        </is>
+      </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="inlineStr">
+        <is>
+          <t>** 02/08 — orden de carpetas y documentos: la cifra 246/105 retirada por no reproducirse. Sin cerrar → 00-direccion/expedientes/07.01.01.md</t>
+        </is>
+      </c>
+      <c r="G77" s="4" t="inlineStr">
+        <is>
+          <t>FICHA (02/08): ALCANCE — cuatro arreglos de documento, NINGUNO toca código: (a) Las celdas ESTADO de 01.02.04 y 03.01.12 declaran en negrita un estado del vocabulario pendiente / en_curso / hecha / bloqueada, como exige la sección «Estados y cadencia de este WBS». Valores ya decididos por el orquestador, no se deducen: 01.02.04 pasa a en_curso (entregado INFORME_MCP_2.md, RECHAZADO por critico-codigo, sin reparar); 03.01.12 pasa a pendiente (nadie la ha trabajado). En 01.02.04 la marca actual […] texto completo en 00-direccion/expedientes/07.01.01.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="13" t="inlineStr">
+        <is>
+          <t>07.01.03</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>NUEVA 03/08 (incidente de proceso): auditar todo lo escrito el 03/08/2026 entre las 21:44 y las 21:58 sin flujo de cuatro capas, y el residuo sin commitear del tramo anterior</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>Orquestador</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="inlineStr">
+        <is>
+          <t>En curso</t>
+        </is>
+      </c>
+      <c r="F78" s="4" t="inlineStr">
+        <is>
+          <t>** 09/08 — auditoria de lo escrito sin flujo el 03/08; los lotes de aptitud cancelados por el CEO → 00-direccion/expedientes/07.01.03.md</t>
+        </is>
+      </c>
+      <c r="G78" s="4" t="inlineStr">
+        <is>
+          <t>FICHA (03/08, dictada por el orquestador): Qué pasó, medido y no supuesto: tras un /compact a las 21:29, la sesión recibió una orden del CEO a las 21:44 y trabajó sola hasta las 21:58 sin invocar a un solo subagente. Escribió D-19, D-20 y D-21 en un registro de solo-añadir, L-024 a L-027, cirugía estructural sobre el WBS, y dos scripts del Excel del CEO. Nadie lo revisó (regla 16 de CLAUDE.md y C2 rotas). Alcance: tres lotes con veredicto propio — (d) procedencia del motor de backtest, (b y c) […] texto completo en 00-direccion/expedientes/07.01.03.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="13" t="inlineStr">
+        <is>
           <t>07.01.02</t>
         </is>
       </c>
-      <c r="B77" s="4" t="inlineStr">
+      <c r="B79" s="4" t="inlineStr">
         <is>
           <t>Mejoras del motor: SOLO tareas aprobadas en revisión semanal (el motor no manda)</t>
         </is>
       </c>
-      <c r="C77" s="4" t="inlineStr">
+      <c r="C79" s="4" t="inlineStr">
         <is>
           <t>Constructores</t>
         </is>
       </c>
-      <c r="D77" s="4" t="inlineStr">
+      <c r="D79" s="4" t="inlineStr">
         <is>
           <t>03.01.02</t>
         </is>
       </c>
-      <c r="E77" s="4" t="inlineStr">
+      <c r="E79" s="4" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F77" s="4" t="inlineStr"/>
-      <c r="G77" s="4" t="inlineStr"/>
+      <c r="F79" s="4" t="inlineStr"/>
+      <c r="G79" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G77"/>
+  <autoFilter ref="A4:G79"/>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <conditionalFormatting sqref="E5:E77">
+  <conditionalFormatting sqref="E5:E79">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Hecha"</formula>
     </cfRule>
@@ -5441,7 +5583,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E5:E77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E5:E79" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pendiente,En curso,Hecha,Bloqueada"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
meta: regenerada la vista Excel del CEO tras los cambios del 12/08
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/05-vista-ceo/WBS_Bot_Trading_v0.9.xlsx
+++ b/05-vista-ceo/WBS_Bot_Trading_v0.9.xlsx
@@ -4400,14 +4400,10 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>** 03/08 — ficha escrita: reparar la prueba 7 del verificador para que examine celdas completas. Sin ejecutar → 00-direccion/expedientes/03.01.17.md</t>
-        </is>
-      </c>
-      <c r="G39" s="4" t="inlineStr">
-        <is>
-          <t>FICHA (03/08): Problema reproducido hoy: la prueba 7 localiza entregables citados en las celdas de tarea, pero corta cada celda por el primer hecha y solo examina lo que va después. En 03.01.13 ese marcador es el último carácter de la celda, así que examina cero ficheros y no caza que esa tarea, marcada hecha, cita 00-direccion/PENDIENTE-03.01.13-lista-de-reglas.md, que no existe en disco ni ha existido nunca en git. Dos defectos más: busca por nombre de fichero en CUALQUIER parte del […] texto completo en 00-direccion/expedientes/03.01.17.md</t>
-        </is>
-      </c>
+          <t>** 03/08 — ficha escrita: reparar la prueba 7 del verificador para que examine celdas completas. La reparacion de la prueba 7 SIGUE sin ejecutar; el 12/08 se ejecuto solo el bloque recortado por el CEO (comprobacion cero en dos fichas + los 9 avisos clasificados) → 00-direccion/expedientes/03.01.17.md</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="13" t="inlineStr">

</xml_diff>